<commit_message>
Backfill ALM ngan hang — Q1-2026 — 2026-09-17
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -31588,7 +31588,7 @@
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>2026-08-31T23:15:14+07:00</t>
+          <t>2026-09-17T09:37:41+07:00</t>
         </is>
       </c>
     </row>
@@ -35625,7 +35625,7 @@
       </c>
       <c r="AH60" t="inlineStr">
         <is>
-          <t>2026-08-31T23:33:10+07:00</t>
+          <t>2026-09-17T09:43:14+07:00</t>
         </is>
       </c>
     </row>
@@ -38215,7 +38215,7 @@
       </c>
       <c r="AH90" t="inlineStr">
         <is>
-          <t>2026-08-31T23:42:53+07:00</t>
+          <t>2026-09-17T09:46:33+07:00</t>
         </is>
       </c>
     </row>
@@ -39669,7 +39669,7 @@
       </c>
       <c r="AH108" t="inlineStr">
         <is>
-          <t>2026-08-31T23:47:32+07:00</t>
+          <t>2026-09-17T09:48:13+07:00</t>
         </is>
       </c>
     </row>
@@ -40775,7 +40775,7 @@
       </c>
       <c r="AH120" t="inlineStr">
         <is>
-          <t>2026-08-31T23:53:52+07:00</t>
+          <t>2026-09-17T09:53:19+07:00</t>
         </is>
       </c>
     </row>
@@ -41583,7 +41583,7 @@
       </c>
       <c r="AH132" t="inlineStr">
         <is>
-          <t>2026-09-01T00:02:09+07:00</t>
+          <t>2026-09-17T09:59:43+07:00</t>
         </is>
       </c>
     </row>
@@ -41931,7 +41931,7 @@
       </c>
       <c r="AH138" t="inlineStr">
         <is>
-          <t>2026-09-01T00:02:19+07:00</t>
+          <t>2026-09-17T09:59:50+07:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bank ALM: nhap thu cong BID 2025-Q1 va STB 2026-Q1/Q2 tu anh chup BCTC that
OCR khong doc duoc du lieu nay (BID: dong "Muc chenh..." nam qua sat dong ghi
chu bi gom nham; STB: chua co bang lai suat trong store dan 2025) - user cung
cap anh chup truc tiep tung trang thuyet minh that, da doi chieu tong 2 chieu
(cong tung dong = cot "Tong", cong tung cot = dong "Tong") khop tuyet doi voi
ca 3 ky truoc khi nhap, danh dau ro nguon la "Nhap thu cong" (khong phai OCR)
de minh bach khi tra cuu lai.
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30918,7 +30918,7 @@
         <v>4.068</v>
       </c>
       <c r="V4" t="n">
-        <v>8183.362999999996</v>
+        <v>8183.362999999999</v>
       </c>
       <c r="W4" t="n">
         <v>-7.633</v>
@@ -31007,7 +31007,7 @@
         <v>3.572</v>
       </c>
       <c r="V5" t="n">
-        <v>-2072.081999999995</v>
+        <v>-2072.081999999999</v>
       </c>
       <c r="W5" t="n">
         <v>-6.467</v>
@@ -31111,7 +31111,7 @@
         <v>4.395</v>
       </c>
       <c r="V6" t="n">
-        <v>-5551.592999999999</v>
+        <v>-5551.593000000001</v>
       </c>
       <c r="W6" t="n">
         <v>0.38</v>
@@ -31408,7 +31408,7 @@
         <v>2.424</v>
       </c>
       <c r="V9" t="n">
-        <v>85041.65799999997</v>
+        <v>85041.658</v>
       </c>
       <c r="W9" t="n">
         <v>-9.567</v>
@@ -32303,12 +32303,98 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>2856110.951</v>
+      </c>
+      <c r="F20" t="n">
+        <v>155906.31</v>
+      </c>
+      <c r="G20" t="n">
+        <v>13945.584</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1976945.954</v>
+      </c>
+      <c r="I20" t="n">
+        <v>2068679.098</v>
+      </c>
+      <c r="J20" t="n">
+        <v>104.64</v>
+      </c>
+      <c r="K20" t="n">
+        <v>419121.4939999999</v>
+      </c>
+      <c r="L20" t="n">
+        <v>-197713.778</v>
+      </c>
+      <c r="M20" t="n">
+        <v>-6.922</v>
+      </c>
+      <c r="N20" t="n">
+        <v>-3.918</v>
+      </c>
+      <c r="O20" t="n">
+        <v>-10.659</v>
+      </c>
+      <c r="P20" t="n">
+        <v>2339610.113</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>861336.583</v>
+      </c>
+      <c r="R20" t="n">
+        <v>271.626</v>
+      </c>
+      <c r="S20" t="n">
+        <v>59.965</v>
+      </c>
+      <c r="T20" t="n">
+        <v>166.764</v>
+      </c>
+      <c r="U20" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="V20" t="n">
+        <v>-169700.807</v>
+      </c>
+      <c r="W20" t="n">
+        <v>-17.588</v>
+      </c>
+      <c r="X20" t="n">
+        <v>-11.033</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>-5.942</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>2718135.967</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>2643816.65</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>102.811</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>-936</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>-6.712</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>Nhap thu cong tu anh chup BCTC that (BID BCTC hop nhat GND Quy I 2025, OCR khong doc duoc)</t>
         </is>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>2026-08-31T16:51:48+07:00</t>
+          <t>2026-09-17T14:38:33+07:00</t>
         </is>
       </c>
     </row>
@@ -32624,7 +32710,7 @@
         <v>2.564</v>
       </c>
       <c r="V26" t="n">
-        <v>-2093.93</v>
+        <v>-2093.930000000001</v>
       </c>
       <c r="W26" t="n">
         <v>0</v>
@@ -33723,7 +33809,7 @@
         <v>584740.964</v>
       </c>
       <c r="L37" t="n">
-        <v>57219.16100000001</v>
+        <v>57219.161</v>
       </c>
       <c r="M37" t="n">
         <v>1.932</v>
@@ -34035,7 +34121,7 @@
         <v>2.439</v>
       </c>
       <c r="V40" t="n">
-        <v>-6843.675999999999</v>
+        <v>-6843.676</v>
       </c>
       <c r="W40" t="n">
         <v>-9.135999999999999</v>
@@ -34213,7 +34299,7 @@
         <v>42408.00799999999</v>
       </c>
       <c r="L42" t="n">
-        <v>2554.764000000001</v>
+        <v>2554.764</v>
       </c>
       <c r="M42" t="n">
         <v>0.946</v>
@@ -34710,7 +34796,7 @@
         <v>3.011</v>
       </c>
       <c r="V49" t="n">
-        <v>1097.082999999999</v>
+        <v>1097.083000000001</v>
       </c>
       <c r="W49" t="n">
         <v>3.244</v>
@@ -36365,7 +36451,7 @@
         <v>53049.641</v>
       </c>
       <c r="L68" t="n">
-        <v>-71627.23300000001</v>
+        <v>-71627.23299999999</v>
       </c>
       <c r="M68" t="n">
         <v>-22.759</v>
@@ -36707,7 +36793,7 @@
         <v>4.335</v>
       </c>
       <c r="V71" t="n">
-        <v>-36336.33499999999</v>
+        <v>-36336.335</v>
       </c>
       <c r="W71" t="n">
         <v>7.502</v>
@@ -36989,7 +37075,7 @@
         <v>3.04</v>
       </c>
       <c r="V74" t="n">
-        <v>1044.137999999999</v>
+        <v>1044.137999999998</v>
       </c>
       <c r="W74" t="n">
         <v>-0.302</v>
@@ -37093,7 +37179,7 @@
         <v>4.485</v>
       </c>
       <c r="V75" t="n">
-        <v>-7342.066000000003</v>
+        <v>-7342.066000000001</v>
       </c>
       <c r="W75" t="n">
         <v>1.12</v>
@@ -37880,7 +37966,7 @@
         <v>3.06</v>
       </c>
       <c r="V83" t="n">
-        <v>44447.072</v>
+        <v>44447.07199999999</v>
       </c>
       <c r="W83" t="n">
         <v>41.067</v>
@@ -38673,7 +38759,7 @@
         <v>6.429</v>
       </c>
       <c r="V95" t="n">
-        <v>-448.712</v>
+        <v>-448.7119999999998</v>
       </c>
       <c r="W95" t="n">
         <v>-8.398</v>
@@ -38955,7 +39041,7 @@
         <v>3.682</v>
       </c>
       <c r="V98" t="n">
-        <v>-8415.234000000002</v>
+        <v>-8415.234</v>
       </c>
       <c r="W98" t="n">
         <v>-5.98</v>
@@ -40770,12 +40856,98 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>859571.527</v>
+      </c>
+      <c r="F120" t="n">
+        <v>61476.611</v>
+      </c>
+      <c r="G120" t="n">
+        <v>6042.042</v>
+      </c>
+      <c r="H120" t="n">
+        <v>600788.965</v>
+      </c>
+      <c r="I120" t="n">
+        <v>604877.709</v>
+      </c>
+      <c r="J120" t="n">
+        <v>100.681</v>
+      </c>
+      <c r="K120" t="n">
+        <v>136075.405</v>
+      </c>
+      <c r="L120" t="n">
+        <v>-53926.931</v>
+      </c>
+      <c r="M120" t="n">
+        <v>-6.274</v>
+      </c>
+      <c r="N120" t="n">
+        <v>-10.42</v>
+      </c>
+      <c r="O120" t="n">
+        <v>-19.247</v>
+      </c>
+      <c r="P120" t="n">
+        <v>776960.677</v>
+      </c>
+      <c r="Q120" t="n">
+        <v>281789.178</v>
+      </c>
+      <c r="R120" t="n">
+        <v>275.724</v>
+      </c>
+      <c r="S120" t="n">
+        <v>29.317</v>
+      </c>
+      <c r="T120" t="n">
+        <v>341.104</v>
+      </c>
+      <c r="U120" t="n">
+        <v>2.265</v>
+      </c>
+      <c r="V120" t="n">
+        <v>-38127.26599999999</v>
+      </c>
+      <c r="W120" t="n">
+        <v>1.911</v>
+      </c>
+      <c r="X120" t="n">
+        <v>27.897</v>
+      </c>
+      <c r="Y120" t="n">
+        <v>-4.436</v>
+      </c>
+      <c r="Z120" t="n">
+        <v>803932.3370000001</v>
+      </c>
+      <c r="AA120" t="n">
+        <v>776334.534</v>
+      </c>
+      <c r="AB120" t="n">
+        <v>103.555</v>
+      </c>
+      <c r="AC120" t="n">
+        <v>659</v>
+      </c>
+      <c r="AD120" t="n">
+        <v>10.907</v>
+      </c>
+      <c r="AE120" t="n">
+        <v>1.072</v>
+      </c>
+      <c r="AF120" t="inlineStr">
+        <is>
+          <t>Nhap thu cong tu anh chup BCTC that (STB BCTC hop nhat GND Quy I 2026, OCR khong doc duoc)</t>
         </is>
       </c>
       <c r="AH120" t="inlineStr">
         <is>
-          <t>2026-09-17T09:53:19+07:00</t>
+          <t>2026-09-17T14:38:33+07:00</t>
         </is>
       </c>
     </row>
@@ -40792,12 +40964,98 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>892048.566</v>
+      </c>
+      <c r="F121" t="n">
+        <v>62807.249</v>
+      </c>
+      <c r="G121" t="n">
+        <v>6247.243</v>
+      </c>
+      <c r="H121" t="n">
+        <v>647939.224</v>
+      </c>
+      <c r="I121" t="n">
+        <v>608851.996</v>
+      </c>
+      <c r="J121" t="n">
+        <v>93.967</v>
+      </c>
+      <c r="K121" t="n">
+        <v>154058.217</v>
+      </c>
+      <c r="L121" t="n">
+        <v>-32668.77299999999</v>
+      </c>
+      <c r="M121" t="n">
+        <v>-3.662</v>
+      </c>
+      <c r="N121" t="n">
+        <v>-5.884</v>
+      </c>
+      <c r="O121" t="n">
+        <v>-14.194</v>
+      </c>
+      <c r="P121" t="n">
+        <v>776523.792</v>
+      </c>
+      <c r="Q121" t="n">
+        <v>280549.491</v>
+      </c>
+      <c r="R121" t="n">
+        <v>276.787</v>
+      </c>
+      <c r="S121" t="n">
+        <v>41.178</v>
+      </c>
+      <c r="T121" t="n">
+        <v>242.848</v>
+      </c>
+      <c r="U121" t="n">
+        <v>2.378</v>
+      </c>
+      <c r="V121" t="n">
+        <v>-7187.399999999994</v>
+      </c>
+      <c r="W121" t="n">
+        <v>2.313</v>
+      </c>
+      <c r="X121" t="n">
+        <v>29.993</v>
+      </c>
+      <c r="Y121" t="n">
+        <v>-0.806</v>
+      </c>
+      <c r="Z121" t="n">
+        <v>820020.6800000001</v>
+      </c>
+      <c r="AA121" t="n">
+        <v>808189.617</v>
+      </c>
+      <c r="AB121" t="n">
+        <v>101.464</v>
+      </c>
+      <c r="AC121" t="n">
+        <v>923</v>
+      </c>
+      <c r="AD121" t="n">
+        <v>14.775</v>
+      </c>
+      <c r="AE121" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="AF121" t="inlineStr">
+        <is>
+          <t>Nhap thu cong tu anh chup BCTC that (STB BCTC hop nhat GND Quy II 2026, OCR khong doc duoc)</t>
         </is>
       </c>
       <c r="AH121" t="inlineStr">
         <is>
-          <t>2026-09-01T10:10:24+07:00</t>
+          <t>2026-09-17T14:38:33+07:00</t>
         </is>
       </c>
     </row>
@@ -41166,7 +41424,7 @@
         <v>3.255</v>
       </c>
       <c r="V125" t="n">
-        <v>-95355.82799999998</v>
+        <v>-95355.82799999999</v>
       </c>
       <c r="W125" t="n">
         <v>-8.385</v>
@@ -41270,7 +41528,7 @@
         <v>3.105</v>
       </c>
       <c r="V126" t="n">
-        <v>31803.23300000001</v>
+        <v>31803.233</v>
       </c>
       <c r="W126" t="n">
         <v>4.369</v>
@@ -41374,7 +41632,7 @@
         <v>2.784</v>
       </c>
       <c r="V127" t="n">
-        <v>49624.19500000001</v>
+        <v>49624.19499999999</v>
       </c>
       <c r="W127" t="n">
         <v>9.231999999999999</v>
@@ -43376,7 +43634,7 @@
         <v>3.722</v>
       </c>
       <c r="V154" t="n">
-        <v>18205.90499999999</v>
+        <v>18205.905</v>
       </c>
       <c r="W154" t="n">
         <v>-11.997</v>

</xml_diff>

<commit_message>
Cap nhat ALM ACB — Q4-2025 — 2026-09-17
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30918,7 +30918,7 @@
         <v>4.068</v>
       </c>
       <c r="V4" t="n">
-        <v>8183.362999999999</v>
+        <v>8183.362999999996</v>
       </c>
       <c r="W4" t="n">
         <v>-7.633</v>
@@ -31007,7 +31007,7 @@
         <v>3.572</v>
       </c>
       <c r="V5" t="n">
-        <v>-2072.081999999999</v>
+        <v>-2072.081999999995</v>
       </c>
       <c r="W5" t="n">
         <v>-6.467</v>
@@ -31111,7 +31111,7 @@
         <v>4.395</v>
       </c>
       <c r="V6" t="n">
-        <v>-5551.593000000001</v>
+        <v>-5551.592999999999</v>
       </c>
       <c r="W6" t="n">
         <v>0.38</v>
@@ -31408,7 +31408,7 @@
         <v>2.424</v>
       </c>
       <c r="V9" t="n">
-        <v>85041.658</v>
+        <v>85041.65799999997</v>
       </c>
       <c r="W9" t="n">
         <v>-9.567</v>
@@ -31561,12 +31561,103 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1025850.127</v>
+      </c>
+      <c r="F11" t="n">
+        <v>94519.719</v>
+      </c>
+      <c r="G11" t="n">
+        <v>7093.272</v>
+      </c>
+      <c r="H11" t="n">
+        <v>585180.175</v>
+      </c>
+      <c r="I11" t="n">
+        <v>679152.623</v>
+      </c>
+      <c r="J11" t="n">
+        <v>116.059</v>
+      </c>
+      <c r="K11" t="n">
+        <v>175190.187</v>
+      </c>
+      <c r="L11" t="n">
+        <v>-36148.089</v>
+      </c>
+      <c r="M11" t="n">
+        <v>-3.524</v>
+      </c>
+      <c r="N11" t="n">
+        <v>-3.551</v>
+      </c>
+      <c r="O11" t="n">
+        <v>-3.553</v>
+      </c>
+      <c r="P11" t="n">
+        <v>39862.162</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>65.181</v>
+      </c>
+      <c r="R11" t="n">
+        <v>61156.107</v>
+      </c>
+      <c r="S11" t="n">
+        <v>206354.522</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="U11" t="n">
+        <v>2.994</v>
+      </c>
+      <c r="V11" t="n">
+        <v>56064.00199999996</v>
+      </c>
+      <c r="W11" t="n">
+        <v>-10.987</v>
+      </c>
+      <c r="X11" t="n">
+        <v>32.032</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>5.465</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>971913.916</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>906469.3540000001</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>107.22</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>1290</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>18.186</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>1.365</v>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất đã kiểm toán năm 2025</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>https://cdn.24hmoney.vn/upload/file/2026-1/2026-03-07/no-name-1772854112.pdf</t>
         </is>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>2026-08-31T01:05:37+07:00</t>
+          <t>2026-09-17T14:57:20+07:00</t>
         </is>
       </c>
     </row>
@@ -32710,7 +32801,7 @@
         <v>2.564</v>
       </c>
       <c r="V26" t="n">
-        <v>-2093.930000000001</v>
+        <v>-2093.93</v>
       </c>
       <c r="W26" t="n">
         <v>0</v>
@@ -33809,7 +33900,7 @@
         <v>584740.964</v>
       </c>
       <c r="L37" t="n">
-        <v>57219.161</v>
+        <v>57219.16100000001</v>
       </c>
       <c r="M37" t="n">
         <v>1.932</v>
@@ -34121,7 +34212,7 @@
         <v>2.439</v>
       </c>
       <c r="V40" t="n">
-        <v>-6843.676</v>
+        <v>-6843.675999999999</v>
       </c>
       <c r="W40" t="n">
         <v>-9.135999999999999</v>
@@ -34299,7 +34390,7 @@
         <v>42408.00799999999</v>
       </c>
       <c r="L42" t="n">
-        <v>2554.764</v>
+        <v>2554.764000000001</v>
       </c>
       <c r="M42" t="n">
         <v>0.946</v>
@@ -34796,7 +34887,7 @@
         <v>3.011</v>
       </c>
       <c r="V49" t="n">
-        <v>1097.083000000001</v>
+        <v>1097.082999999999</v>
       </c>
       <c r="W49" t="n">
         <v>3.244</v>
@@ -36451,7 +36542,7 @@
         <v>53049.641</v>
       </c>
       <c r="L68" t="n">
-        <v>-71627.23299999999</v>
+        <v>-71627.23300000001</v>
       </c>
       <c r="M68" t="n">
         <v>-22.759</v>
@@ -36793,7 +36884,7 @@
         <v>4.335</v>
       </c>
       <c r="V71" t="n">
-        <v>-36336.335</v>
+        <v>-36336.33499999999</v>
       </c>
       <c r="W71" t="n">
         <v>7.502</v>
@@ -37075,7 +37166,7 @@
         <v>3.04</v>
       </c>
       <c r="V74" t="n">
-        <v>1044.137999999998</v>
+        <v>1044.137999999999</v>
       </c>
       <c r="W74" t="n">
         <v>-0.302</v>
@@ -37179,7 +37270,7 @@
         <v>4.485</v>
       </c>
       <c r="V75" t="n">
-        <v>-7342.066000000001</v>
+        <v>-7342.066000000003</v>
       </c>
       <c r="W75" t="n">
         <v>1.12</v>
@@ -37966,7 +38057,7 @@
         <v>3.06</v>
       </c>
       <c r="V83" t="n">
-        <v>44447.07199999999</v>
+        <v>44447.072</v>
       </c>
       <c r="W83" t="n">
         <v>41.067</v>
@@ -38759,7 +38850,7 @@
         <v>6.429</v>
       </c>
       <c r="V95" t="n">
-        <v>-448.7119999999998</v>
+        <v>-448.712</v>
       </c>
       <c r="W95" t="n">
         <v>-8.398</v>
@@ -39041,7 +39132,7 @@
         <v>3.682</v>
       </c>
       <c r="V98" t="n">
-        <v>-8415.234</v>
+        <v>-8415.234000000002</v>
       </c>
       <c r="W98" t="n">
         <v>-5.98</v>
@@ -41424,7 +41515,7 @@
         <v>3.255</v>
       </c>
       <c r="V125" t="n">
-        <v>-95355.82799999999</v>
+        <v>-95355.82799999998</v>
       </c>
       <c r="W125" t="n">
         <v>-8.385</v>
@@ -41528,7 +41619,7 @@
         <v>3.105</v>
       </c>
       <c r="V126" t="n">
-        <v>31803.233</v>
+        <v>31803.23300000001</v>
       </c>
       <c r="W126" t="n">
         <v>4.369</v>
@@ -41632,7 +41723,7 @@
         <v>2.784</v>
       </c>
       <c r="V127" t="n">
-        <v>49624.19499999999</v>
+        <v>49624.19500000001</v>
       </c>
       <c r="W127" t="n">
         <v>9.231999999999999</v>
@@ -43634,7 +43725,7 @@
         <v>3.722</v>
       </c>
       <c r="V154" t="n">
-        <v>18205.905</v>
+        <v>18205.90499999999</v>
       </c>
       <c r="W154" t="n">
         <v>-11.997</v>

</xml_diff>

<commit_message>
Cap nhat ALM ACB — q1-2026 — 2026-09-17
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -31674,12 +31674,94 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1030900.741</v>
+      </c>
+      <c r="F12" t="n">
+        <v>98751.052</v>
+      </c>
+      <c r="G12" t="n">
+        <v>6989.162</v>
+      </c>
+      <c r="H12" t="n">
+        <v>569109.608</v>
+      </c>
+      <c r="I12" t="n">
+        <v>701211.785</v>
+      </c>
+      <c r="J12" t="n">
+        <v>123.212</v>
+      </c>
+      <c r="K12" t="n">
+        <v>156854.572</v>
+      </c>
+      <c r="L12" t="n">
+        <v>-271.2610000000001</v>
+      </c>
+      <c r="M12" t="n">
+        <v>-0.026</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="P12" t="n">
+        <v>49924.416</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>51216.558</v>
+      </c>
+      <c r="R12" t="n">
+        <v>97.477</v>
+      </c>
+      <c r="S12" t="n">
+        <v>193.815</v>
+      </c>
+      <c r="T12" t="n">
+        <v>51.596</v>
+      </c>
+      <c r="U12" t="n">
+        <v>2.756</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20260422_-_ACB_-_BCTC_Hop_nhat_Quy_1_nam_2026_1776932823.pdf</t>
         </is>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>2026-09-17T09:37:41+07:00</t>
+          <t>2026-09-17T15:01:42+07:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cap nhat ALM BID — Q2-2025 — 2026-09-17
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -32584,12 +32584,88 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>2991644.165</v>
+      </c>
+      <c r="F21" t="n">
+        <v>162737.31</v>
+      </c>
+      <c r="G21" t="n">
+        <v>14991.731</v>
+      </c>
+      <c r="H21" t="n">
+        <v>2074787.517</v>
+      </c>
+      <c r="I21" t="n">
+        <v>2141443.805</v>
+      </c>
+      <c r="J21" t="n">
+        <v>103.213</v>
+      </c>
+      <c r="K21" t="n">
+        <v>486478.838</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" t="n">
+        <v>2.345</v>
+      </c>
+      <c r="V21" t="n">
+        <v>-677107.5850000001</v>
+      </c>
+      <c r="W21" t="n">
+        <v>-25.843</v>
+      </c>
+      <c r="X21" t="n">
+        <v>-8.513999999999999</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>-22.633</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>569385.233</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>1301394.451</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>43.752</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>-4094</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>-27.308</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>-2.516</v>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/BID_Baocaotaichinh_6T_2025_Soatxet_Hopnhat_03102025143111.pdf</t>
         </is>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>2026-08-31T11:50:13+07:00</t>
+          <t>2026-09-17T15:06:22+07:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cap nhat ALM cac ma dang missing — q1-2025 — 2026-09-17
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -38462,7 +38462,7 @@
       </c>
       <c r="AH86" t="inlineStr">
         <is>
-          <t>2026-08-31T16:58:48+07:00</t>
+          <t>2026-09-17T15:23:31+07:00</t>
         </is>
       </c>
     </row>
@@ -39834,7 +39834,7 @@
       </c>
       <c r="AH104" t="inlineStr">
         <is>
-          <t>2026-08-31T17:00:11+07:00</t>
+          <t>2026-09-17T15:24:51+07:00</t>
         </is>
       </c>
     </row>
@@ -41930,12 +41930,103 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>388891.15</v>
+      </c>
+      <c r="F128" t="n">
+        <v>39491.596</v>
+      </c>
+      <c r="G128" t="n">
+        <v>3383.618</v>
+      </c>
+      <c r="H128" t="n">
+        <v>233114.646</v>
+      </c>
+      <c r="I128" t="n">
+        <v>259070.461</v>
+      </c>
+      <c r="J128" t="n">
+        <v>111.134</v>
+      </c>
+      <c r="K128" t="n">
+        <v>53519.87700000001</v>
+      </c>
+      <c r="L128" t="n">
+        <v>1173.397999999997</v>
+      </c>
+      <c r="M128" t="n">
+        <v>0.302</v>
+      </c>
+      <c r="N128" t="n">
+        <v>0.283</v>
+      </c>
+      <c r="O128" t="n">
+        <v>0.323</v>
+      </c>
+      <c r="P128" t="n">
+        <v>29361.059</v>
+      </c>
+      <c r="Q128" t="n">
+        <v>206.249</v>
+      </c>
+      <c r="R128" t="n">
+        <v>14235.734</v>
+      </c>
+      <c r="S128" t="n">
+        <v>19232.121</v>
+      </c>
+      <c r="T128" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="U128" t="n">
+        <v>2.296</v>
+      </c>
+      <c r="V128" t="n">
+        <v>47597.061</v>
+      </c>
+      <c r="W128" t="n">
+        <v>12.611</v>
+      </c>
+      <c r="X128" t="n">
+        <v>12.468</v>
+      </c>
+      <c r="Y128" t="n">
+        <v>12.239</v>
+      </c>
+      <c r="Z128" t="n">
+        <v>62861.954</v>
+      </c>
+      <c r="AA128" t="n">
+        <v>35233.365</v>
+      </c>
+      <c r="AB128" t="n">
+        <v>178.416</v>
+      </c>
+      <c r="AC128" t="n">
+        <v>461</v>
+      </c>
+      <c r="AD128" t="n">
+        <v>13.624</v>
+      </c>
+      <c r="AE128" t="n">
+        <v>1.167</v>
+      </c>
+      <c r="AF128" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="AG128" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/TPB_Baocaotaichinh_Q1_2025_Hopnhat_23052025145349.pdf</t>
         </is>
       </c>
       <c r="AH128" t="inlineStr">
         <is>
-          <t>2026-08-31T17:05:53+07:00</t>
+          <t>2026-09-17T15:27:28+07:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bank ALM: nhap thu cong OCB 2025-Q1 tu anh chup BCTC that (don vi VND, da quy doi)
OCB cong bo bao cao bang don vi VND THUC (khong phai "Trieu dong" nhu hau het
cac ngan hang khac) - da chia 1.000.000 de quy doi ve "trieu dong" truoc khi
luu, khop quy uoc chung cua he thong. Da doi chieu voi quarterly_balance_sheet
doc lap tu Vietcap (291.551 ty tu bang gap vs 289.067 ty tu Vietcap, lech
~0.85%, hop ly) de xac nhan quy doi dung don vi truoc khi nhap.
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30918,7 +30918,7 @@
         <v>4.068</v>
       </c>
       <c r="V4" t="n">
-        <v>8183.362999999996</v>
+        <v>8183.362999999999</v>
       </c>
       <c r="W4" t="n">
         <v>-7.633</v>
@@ -31007,7 +31007,7 @@
         <v>3.572</v>
       </c>
       <c r="V5" t="n">
-        <v>-2072.081999999995</v>
+        <v>-2072.081999999999</v>
       </c>
       <c r="W5" t="n">
         <v>-6.467</v>
@@ -31111,7 +31111,7 @@
         <v>4.395</v>
       </c>
       <c r="V6" t="n">
-        <v>-5551.592999999999</v>
+        <v>-5551.593000000001</v>
       </c>
       <c r="W6" t="n">
         <v>0.38</v>
@@ -31408,7 +31408,7 @@
         <v>2.424</v>
       </c>
       <c r="V9" t="n">
-        <v>85041.65799999997</v>
+        <v>85041.658</v>
       </c>
       <c r="W9" t="n">
         <v>-9.567</v>
@@ -32959,7 +32959,7 @@
         <v>2.564</v>
       </c>
       <c r="V26" t="n">
-        <v>-2093.93</v>
+        <v>-2093.930000000001</v>
       </c>
       <c r="W26" t="n">
         <v>0</v>
@@ -34058,7 +34058,7 @@
         <v>584740.964</v>
       </c>
       <c r="L37" t="n">
-        <v>57219.16100000001</v>
+        <v>57219.161</v>
       </c>
       <c r="M37" t="n">
         <v>1.932</v>
@@ -34370,7 +34370,7 @@
         <v>2.439</v>
       </c>
       <c r="V40" t="n">
-        <v>-6843.675999999999</v>
+        <v>-6843.676</v>
       </c>
       <c r="W40" t="n">
         <v>-9.135999999999999</v>
@@ -34548,7 +34548,7 @@
         <v>42408.00799999999</v>
       </c>
       <c r="L42" t="n">
-        <v>2554.764000000001</v>
+        <v>2554.764</v>
       </c>
       <c r="M42" t="n">
         <v>0.946</v>
@@ -35045,7 +35045,7 @@
         <v>3.011</v>
       </c>
       <c r="V49" t="n">
-        <v>1097.082999999999</v>
+        <v>1097.083000000001</v>
       </c>
       <c r="W49" t="n">
         <v>3.244</v>
@@ -36700,7 +36700,7 @@
         <v>53049.641</v>
       </c>
       <c r="L68" t="n">
-        <v>-71627.23300000001</v>
+        <v>-71627.23299999999</v>
       </c>
       <c r="M68" t="n">
         <v>-22.759</v>
@@ -37042,7 +37042,7 @@
         <v>4.335</v>
       </c>
       <c r="V71" t="n">
-        <v>-36336.33499999999</v>
+        <v>-36336.335</v>
       </c>
       <c r="W71" t="n">
         <v>7.502</v>
@@ -37324,7 +37324,7 @@
         <v>3.04</v>
       </c>
       <c r="V74" t="n">
-        <v>1044.137999999999</v>
+        <v>1044.137999999998</v>
       </c>
       <c r="W74" t="n">
         <v>-0.302</v>
@@ -37428,7 +37428,7 @@
         <v>4.485</v>
       </c>
       <c r="V75" t="n">
-        <v>-7342.066000000003</v>
+        <v>-7342.066000000001</v>
       </c>
       <c r="W75" t="n">
         <v>1.12</v>
@@ -38215,7 +38215,7 @@
         <v>3.06</v>
       </c>
       <c r="V83" t="n">
-        <v>44447.072</v>
+        <v>44447.07199999999</v>
       </c>
       <c r="W83" t="n">
         <v>41.067</v>
@@ -38457,12 +38457,98 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>289066.935913466</v>
+      </c>
+      <c r="F86" t="n">
+        <v>32388.218496367</v>
+      </c>
+      <c r="G86" t="n">
+        <v>2163.56288338</v>
+      </c>
+      <c r="H86" t="n">
+        <v>151153.873885092</v>
+      </c>
+      <c r="I86" t="n">
+        <v>172738.829352774</v>
+      </c>
+      <c r="J86" t="n">
+        <v>114.28</v>
+      </c>
+      <c r="K86" t="n">
+        <v>40416.050727173</v>
+      </c>
+      <c r="L86" t="n">
+        <v>-40096.556</v>
+      </c>
+      <c r="M86" t="n">
+        <v>-13.871</v>
+      </c>
+      <c r="N86" t="n">
+        <v>-19.78</v>
+      </c>
+      <c r="O86" t="n">
+        <v>-27.062</v>
+      </c>
+      <c r="P86" t="n">
+        <v>214942.078</v>
+      </c>
+      <c r="Q86" t="n">
+        <v>154835.187</v>
+      </c>
+      <c r="R86" t="n">
+        <v>138.82</v>
+      </c>
+      <c r="S86" t="n">
+        <v>47.873</v>
+      </c>
+      <c r="T86" t="n">
+        <v>208.886</v>
+      </c>
+      <c r="U86" t="n">
+        <v>2.674</v>
+      </c>
+      <c r="V86" t="n">
+        <v>31866.49299999999</v>
+      </c>
+      <c r="W86" t="n">
+        <v>-11.425</v>
+      </c>
+      <c r="X86" t="n">
+        <v>-4.928</v>
+      </c>
+      <c r="Y86" t="n">
+        <v>11.024</v>
+      </c>
+      <c r="Z86" t="n">
+        <v>266228.092</v>
+      </c>
+      <c r="AA86" t="n">
+        <v>247087.747</v>
+      </c>
+      <c r="AB86" t="n">
+        <v>107.746</v>
+      </c>
+      <c r="AC86" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD86" t="n">
+        <v>1.849</v>
+      </c>
+      <c r="AE86" t="n">
+        <v>0.124</v>
+      </c>
+      <c r="AF86" t="inlineStr">
+        <is>
+          <t>Nhap thu cong tu anh chup BCTC that (OCB thuyet minh BCTC hop nhat Quy 1 2025, OCR khong doc duoc - don vi VND thuc, da quy doi ve trieu dong)</t>
         </is>
       </c>
       <c r="AH86" t="inlineStr">
         <is>
-          <t>2026-09-17T15:38:57+07:00</t>
+          <t>2026-09-17T16:12:36+07:00</t>
         </is>
       </c>
     </row>
@@ -39008,7 +39094,7 @@
         <v>6.429</v>
       </c>
       <c r="V95" t="n">
-        <v>-448.712</v>
+        <v>-448.7119999999998</v>
       </c>
       <c r="W95" t="n">
         <v>-8.398</v>
@@ -39290,7 +39376,7 @@
         <v>3.682</v>
       </c>
       <c r="V98" t="n">
-        <v>-8415.234000000002</v>
+        <v>-8415.234</v>
       </c>
       <c r="W98" t="n">
         <v>-5.98</v>
@@ -41673,7 +41759,7 @@
         <v>3.255</v>
       </c>
       <c r="V125" t="n">
-        <v>-95355.82799999998</v>
+        <v>-95355.82799999999</v>
       </c>
       <c r="W125" t="n">
         <v>-8.385</v>
@@ -41777,7 +41863,7 @@
         <v>3.105</v>
       </c>
       <c r="V126" t="n">
-        <v>31803.23300000001</v>
+        <v>31803.233</v>
       </c>
       <c r="W126" t="n">
         <v>4.369</v>
@@ -41881,7 +41967,7 @@
         <v>2.784</v>
       </c>
       <c r="V127" t="n">
-        <v>49624.19500000001</v>
+        <v>49624.19499999999</v>
       </c>
       <c r="W127" t="n">
         <v>9.231999999999999</v>
@@ -41985,7 +42071,7 @@
         <v>2.296</v>
       </c>
       <c r="V128" t="n">
-        <v>47597.061</v>
+        <v>47597.06099999999</v>
       </c>
       <c r="W128" t="n">
         <v>12.611</v>
@@ -43974,7 +44060,7 @@
         <v>3.722</v>
       </c>
       <c r="V154" t="n">
-        <v>18205.90499999999</v>
+        <v>18205.905</v>
       </c>
       <c r="W154" t="n">
         <v>-11.997</v>

</xml_diff>

<commit_message>
Cap nhat ALM cac ma dang missing — Q2-2025 — 2026-09-17
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -34835,12 +34835,103 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>784096.287</v>
+      </c>
+      <c r="F45" t="n">
+        <v>64626.363</v>
+      </c>
+      <c r="G45" t="n">
+        <v>9819.157999999999</v>
+      </c>
+      <c r="H45" t="n">
+        <v>478700.229</v>
+      </c>
+      <c r="I45" t="n">
+        <v>502451.955</v>
+      </c>
+      <c r="J45" t="n">
+        <v>104.962</v>
+      </c>
+      <c r="K45" t="n">
+        <v>145778.24</v>
+      </c>
+      <c r="L45" t="n">
+        <v>1318.71</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="N45" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="P45" t="n">
+        <v>348514.834</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>113472.208</v>
+      </c>
+      <c r="R45" t="n">
+        <v>307.137</v>
+      </c>
+      <c r="S45" t="n">
+        <v>156.953</v>
+      </c>
+      <c r="T45" t="n">
+        <v>63.713</v>
+      </c>
+      <c r="U45" t="n">
+        <v>3.045</v>
+      </c>
+      <c r="V45" t="n">
+        <v>172001.015</v>
+      </c>
+      <c r="W45" t="n">
+        <v>0.389</v>
+      </c>
+      <c r="X45" t="n">
+        <v>4.299</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>21.936</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>1435902.857</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>1263818.771</v>
+      </c>
+      <c r="AB45" t="n">
+        <v>113.616</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>871</v>
+      </c>
+      <c r="AD45" t="n">
+        <v>8.869999999999999</v>
+      </c>
+      <c r="AE45" t="n">
+        <v>1.348</v>
+      </c>
+      <c r="AF45" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="AG45" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/HDB_Baocaotaichinh_6T_2025_Soatxet_Hopnhat_03102025151254.pdf</t>
         </is>
       </c>
       <c r="AH45" t="inlineStr">
         <is>
-          <t>2026-08-31T12:01:17+07:00</t>
+          <t>2026-09-17T16:27:10+07:00</t>
         </is>
       </c>
     </row>
@@ -35822,12 +35913,103 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>513612.864</v>
+      </c>
+      <c r="F57" t="n">
+        <v>40699.872</v>
+      </c>
+      <c r="G57" t="n">
+        <v>3735.854</v>
+      </c>
+      <c r="H57" t="n">
+        <v>313174.113</v>
+      </c>
+      <c r="I57" t="n">
+        <v>363890.539</v>
+      </c>
+      <c r="J57" t="n">
+        <v>116.194</v>
+      </c>
+      <c r="K57" t="n">
+        <v>82889.34299999999</v>
+      </c>
+      <c r="L57" t="n">
+        <v>3650.622</v>
+      </c>
+      <c r="M57" t="n">
+        <v>0.711</v>
+      </c>
+      <c r="N57" t="n">
+        <v>0.961</v>
+      </c>
+      <c r="O57" t="n">
+        <v>12.42</v>
+      </c>
+      <c r="P57" t="n">
+        <v>853290.689</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>57642.309</v>
+      </c>
+      <c r="R57" t="n">
+        <v>1480.32</v>
+      </c>
+      <c r="S57" t="n">
+        <v>76.93300000000001</v>
+      </c>
+      <c r="T57" t="n">
+        <v>129.983</v>
+      </c>
+      <c r="U57" t="n">
+        <v>2.647</v>
+      </c>
+      <c r="V57" t="n">
+        <v>-30007.58</v>
+      </c>
+      <c r="W57" t="n">
+        <v>3.512</v>
+      </c>
+      <c r="X57" t="n">
+        <v>7.024</v>
+      </c>
+      <c r="Y57" t="n">
+        <v>-5.842</v>
+      </c>
+      <c r="Z57" t="n">
+        <v>495717.531</v>
+      </c>
+      <c r="AA57" t="n">
+        <v>345939.057</v>
+      </c>
+      <c r="AB57" t="n">
+        <v>143.296</v>
+      </c>
+      <c r="AC57" t="n">
+        <v>-59</v>
+      </c>
+      <c r="AD57" t="n">
+        <v>-1.579</v>
+      </c>
+      <c r="AE57" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="AF57" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="AG57" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/LPB_Baocaotaichinh_6T_2025_Soatxet_06102025090900.pdf</t>
         </is>
       </c>
       <c r="AH57" t="inlineStr">
         <is>
-          <t>2026-08-31T12:07:34+07:00</t>
+          <t>2026-09-17T16:28:03+07:00</t>
         </is>
       </c>
     </row>
@@ -38570,7 +38752,7 @@
       </c>
       <c r="AH87" t="inlineStr">
         <is>
-          <t>2026-08-31T12:23:24+07:00</t>
+          <t>2026-09-17T16:31:33+07:00</t>
         </is>
       </c>
     </row>
@@ -42129,12 +42311,103 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>428589.979</v>
+      </c>
+      <c r="F129" t="n">
+        <v>38229.908</v>
+      </c>
+      <c r="G129" t="n">
+        <v>3151.325</v>
+      </c>
+      <c r="H129" t="n">
+        <v>246844.312</v>
+      </c>
+      <c r="I129" t="n">
+        <v>281188.723</v>
+      </c>
+      <c r="J129" t="n">
+        <v>113.913</v>
+      </c>
+      <c r="K129" t="n">
+        <v>71542.25599999999</v>
+      </c>
+      <c r="L129" t="n">
+        <v>-68400.776</v>
+      </c>
+      <c r="M129" t="n">
+        <v>-15.959</v>
+      </c>
+      <c r="N129" t="n">
+        <v>-17.579</v>
+      </c>
+      <c r="O129" t="n">
+        <v>-17.575</v>
+      </c>
+      <c r="P129" t="n">
+        <v>322684.431</v>
+      </c>
+      <c r="Q129" t="n">
+        <v>164687.777</v>
+      </c>
+      <c r="R129" t="n">
+        <v>195.937</v>
+      </c>
+      <c r="S129" t="n">
+        <v>64.307</v>
+      </c>
+      <c r="T129" t="n">
+        <v>155.504</v>
+      </c>
+      <c r="U129" t="n">
+        <v>2.898</v>
+      </c>
+      <c r="V129" t="n">
+        <v>-23865.841</v>
+      </c>
+      <c r="W129" t="n">
+        <v>0</v>
+      </c>
+      <c r="X129" t="n">
+        <v>4.669</v>
+      </c>
+      <c r="Y129" t="n">
+        <v>-5.568</v>
+      </c>
+      <c r="Z129" t="n">
+        <v>846378.6310000001</v>
+      </c>
+      <c r="AA129" t="n">
+        <v>898757.455</v>
+      </c>
+      <c r="AB129" t="n">
+        <v>94.172</v>
+      </c>
+      <c r="AC129" t="n">
+        <v>82</v>
+      </c>
+      <c r="AD129" t="n">
+        <v>2.602</v>
+      </c>
+      <c r="AE129" t="n">
+        <v>0.214</v>
+      </c>
+      <c r="AF129" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="AG129" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/TPB_Baocaotaichinh_6T_2025_Soatxet_Hopnhat_06102025102458.pdf</t>
         </is>
       </c>
       <c r="AH129" t="inlineStr">
         <is>
-          <t>2026-08-31T12:42:52+07:00</t>
+          <t>2026-09-17T16:32:56+07:00</t>
         </is>
       </c>
     </row>
@@ -42462,12 +42735,88 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>133951.803544459</v>
+      </c>
+      <c r="F135" t="n">
+        <v>9420.642668476999</v>
+      </c>
+      <c r="G135" t="n">
+        <v>542.378510292</v>
+      </c>
+      <c r="H135" t="n">
+        <v>95784.767789663</v>
+      </c>
+      <c r="I135" t="n">
+        <v>86563.862420006</v>
+      </c>
+      <c r="J135" t="n">
+        <v>90.373</v>
+      </c>
+      <c r="K135" t="n">
+        <v>19972.595116502</v>
+      </c>
+      <c r="L135" t="n">
+        <v>0</v>
+      </c>
+      <c r="M135" t="n">
+        <v>0</v>
+      </c>
+      <c r="N135" t="n">
+        <v>0</v>
+      </c>
+      <c r="O135" t="n">
+        <v>0</v>
+      </c>
+      <c r="U135" t="n">
+        <v>2.085</v>
+      </c>
+      <c r="V135" t="n">
+        <v>-28908.298</v>
+      </c>
+      <c r="W135" t="n">
+        <v>0</v>
+      </c>
+      <c r="X135" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y135" t="n">
+        <v>-21.581</v>
+      </c>
+      <c r="Z135" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA135" t="n">
+        <v>28914.298</v>
+      </c>
+      <c r="AB135" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC135" t="n">
+        <v>-126</v>
+      </c>
+      <c r="AD135" t="n">
+        <v>-23.231</v>
+      </c>
+      <c r="AE135" t="n">
+        <v>-1.337</v>
+      </c>
+      <c r="AF135" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025</t>
+        </is>
+      </c>
+      <c r="AG135" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/000007054673721340387ngn-hng-tmcp-vit-24072025-000000bo-co-ti-chnh-hp-nht-qu_1_0914.pdf</t>
         </is>
       </c>
       <c r="AH135" t="inlineStr">
         <is>
-          <t>2026-08-31T12:46:28+07:00</t>
+          <t>2026-09-17T16:34:18+07:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bank ALM: nhap thu cong OCB 2025-Q2 - xac nhan OCB cong bo bang tieng Anh that ky nay
Dieu tra sau khi user bao van loi du bao cao that co du: tai truc tiep CA 3
candidate that cua OCB Quy 2/2025 (nho fix cache o commit 6444c57, moi
candidate gio co file rieng, khong con dung do). Ca 3 deu la ban TIENG ANH
("NOTES TO THE CONSOLIDATED FINANCIAL STATEMENTS") - khac Quy 1/2025 (candidate
24hmoney la tieng Viet). Xac nhan OCB THAT SU cong bo ca 2 ngon ngu tuy ky,
khong phai loi tim kiem.

Doc truc tiep bang anh (khong OCR, doc bang mat qua Read tool) trang 23.1
Interest rate risk + 23.3 Liquidity risk (ca 2 deu don vi VND thuc) - da doi
chieu 2 chieu (tong dong = cot Total, tong cot = dong Total) khop tuyet doi,
va doi chieu voi quarterly_balance_sheet doc lap tu Vietcap (308.899 ty vs
311.600 ty tu bang gap sau quy doi, lech ~0.87%, hop ly) truoc khi nhap.
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30918,7 +30918,7 @@
         <v>4.068</v>
       </c>
       <c r="V4" t="n">
-        <v>8183.362999999996</v>
+        <v>8183.362999999999</v>
       </c>
       <c r="W4" t="n">
         <v>-7.633</v>
@@ -31007,7 +31007,7 @@
         <v>3.572</v>
       </c>
       <c r="V5" t="n">
-        <v>-2072.081999999995</v>
+        <v>-2072.081999999999</v>
       </c>
       <c r="W5" t="n">
         <v>-6.467</v>
@@ -31111,7 +31111,7 @@
         <v>4.395</v>
       </c>
       <c r="V6" t="n">
-        <v>-5551.592999999999</v>
+        <v>-5551.593000000001</v>
       </c>
       <c r="W6" t="n">
         <v>0.38</v>
@@ -31408,7 +31408,7 @@
         <v>2.424</v>
       </c>
       <c r="V9" t="n">
-        <v>85041.65799999997</v>
+        <v>85041.658</v>
       </c>
       <c r="W9" t="n">
         <v>-9.567</v>
@@ -32959,7 +32959,7 @@
         <v>2.564</v>
       </c>
       <c r="V26" t="n">
-        <v>-2093.93</v>
+        <v>-2093.930000000001</v>
       </c>
       <c r="W26" t="n">
         <v>0</v>
@@ -34058,7 +34058,7 @@
         <v>584740.964</v>
       </c>
       <c r="L37" t="n">
-        <v>57219.16100000001</v>
+        <v>57219.161</v>
       </c>
       <c r="M37" t="n">
         <v>1.932</v>
@@ -34370,7 +34370,7 @@
         <v>2.439</v>
       </c>
       <c r="V40" t="n">
-        <v>-6843.675999999999</v>
+        <v>-6843.676</v>
       </c>
       <c r="W40" t="n">
         <v>-9.135999999999999</v>
@@ -34548,7 +34548,7 @@
         <v>42408.00799999999</v>
       </c>
       <c r="L42" t="n">
-        <v>2554.764000000001</v>
+        <v>2554.764</v>
       </c>
       <c r="M42" t="n">
         <v>0.946</v>
@@ -35136,7 +35136,7 @@
         <v>3.011</v>
       </c>
       <c r="V49" t="n">
-        <v>1097.082999999999</v>
+        <v>1097.083000000001</v>
       </c>
       <c r="W49" t="n">
         <v>3.244</v>
@@ -36882,7 +36882,7 @@
         <v>53049.641</v>
       </c>
       <c r="L68" t="n">
-        <v>-71627.23300000001</v>
+        <v>-71627.23299999999</v>
       </c>
       <c r="M68" t="n">
         <v>-22.759</v>
@@ -37224,7 +37224,7 @@
         <v>4.335</v>
       </c>
       <c r="V71" t="n">
-        <v>-36336.33499999999</v>
+        <v>-36336.335</v>
       </c>
       <c r="W71" t="n">
         <v>7.502</v>
@@ -37506,7 +37506,7 @@
         <v>3.04</v>
       </c>
       <c r="V74" t="n">
-        <v>1044.137999999999</v>
+        <v>1044.137999999998</v>
       </c>
       <c r="W74" t="n">
         <v>-0.302</v>
@@ -37610,7 +37610,7 @@
         <v>4.485</v>
       </c>
       <c r="V75" t="n">
-        <v>-7342.066000000003</v>
+        <v>-7342.066000000001</v>
       </c>
       <c r="W75" t="n">
         <v>1.12</v>
@@ -38397,7 +38397,7 @@
         <v>3.06</v>
       </c>
       <c r="V83" t="n">
-        <v>44447.072</v>
+        <v>44447.07199999999</v>
       </c>
       <c r="W83" t="n">
         <v>41.067</v>
@@ -38747,12 +38747,98 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>308899.421013687</v>
+      </c>
+      <c r="F87" t="n">
+        <v>33113.733211965</v>
+      </c>
+      <c r="G87" t="n">
+        <v>2179.122847119</v>
+      </c>
+      <c r="H87" t="n">
+        <v>153939.669388207</v>
+      </c>
+      <c r="I87" t="n">
+        <v>183717.021936619</v>
+      </c>
+      <c r="J87" t="n">
+        <v>119.344</v>
+      </c>
+      <c r="K87" t="n">
+        <v>52580.40211333201</v>
+      </c>
+      <c r="L87" t="n">
+        <v>-54108.582</v>
+      </c>
+      <c r="M87" t="n">
+        <v>-17.517</v>
+      </c>
+      <c r="N87" t="n">
+        <v>-21.187</v>
+      </c>
+      <c r="O87" t="n">
+        <v>-22.834</v>
+      </c>
+      <c r="P87" t="n">
+        <v>224061.667</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>158073.753</v>
+      </c>
+      <c r="R87" t="n">
+        <v>141.745</v>
+      </c>
+      <c r="S87" t="n">
+        <v>53.67</v>
+      </c>
+      <c r="T87" t="n">
+        <v>186.325</v>
+      </c>
+      <c r="U87" t="n">
+        <v>3.416</v>
+      </c>
+      <c r="V87" t="n">
+        <v>36655.177</v>
+      </c>
+      <c r="W87" t="n">
+        <v>-14.516</v>
+      </c>
+      <c r="X87" t="n">
+        <v>-4.869</v>
+      </c>
+      <c r="Y87" t="n">
+        <v>11.866</v>
+      </c>
+      <c r="Z87" t="n">
+        <v>287379.692</v>
+      </c>
+      <c r="AA87" t="n">
+        <v>270403.116</v>
+      </c>
+      <c r="AB87" t="n">
+        <v>106.278</v>
+      </c>
+      <c r="AC87" t="n">
+        <v>59</v>
+      </c>
+      <c r="AD87" t="n">
+        <v>2.708</v>
+      </c>
+      <c r="AE87" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="AF87" t="inlineStr">
+        <is>
+          <t>Nhap thu cong tu doc truc tiep BCTC that (OCB thuyet minh BCTC hop nhat Quy 2 2025, ban tieng Anh, don vi VND thuc da quy doi ve trieu dong, OCR khong doc duoc do bao cao tieng Anh)</t>
         </is>
       </c>
       <c r="AH87" t="inlineStr">
         <is>
-          <t>2026-09-17T16:31:33+07:00</t>
+          <t>2026-09-17T16:58:29+07:00</t>
         </is>
       </c>
     </row>
@@ -39276,7 +39362,7 @@
         <v>6.429</v>
       </c>
       <c r="V95" t="n">
-        <v>-448.712</v>
+        <v>-448.7119999999998</v>
       </c>
       <c r="W95" t="n">
         <v>-8.398</v>
@@ -39558,7 +39644,7 @@
         <v>3.682</v>
       </c>
       <c r="V98" t="n">
-        <v>-8415.234000000002</v>
+        <v>-8415.234</v>
       </c>
       <c r="W98" t="n">
         <v>-5.98</v>
@@ -41941,7 +42027,7 @@
         <v>3.255</v>
       </c>
       <c r="V125" t="n">
-        <v>-95355.82799999998</v>
+        <v>-95355.82799999999</v>
       </c>
       <c r="W125" t="n">
         <v>-8.385</v>
@@ -42045,7 +42131,7 @@
         <v>3.105</v>
       </c>
       <c r="V126" t="n">
-        <v>31803.23300000001</v>
+        <v>31803.233</v>
       </c>
       <c r="W126" t="n">
         <v>4.369</v>
@@ -42149,7 +42235,7 @@
         <v>2.784</v>
       </c>
       <c r="V127" t="n">
-        <v>49624.19500000001</v>
+        <v>49624.19499999999</v>
       </c>
       <c r="W127" t="n">
         <v>9.231999999999999</v>
@@ -42253,7 +42339,7 @@
         <v>2.296</v>
       </c>
       <c r="V128" t="n">
-        <v>47597.061</v>
+        <v>47597.06099999999</v>
       </c>
       <c r="W128" t="n">
         <v>12.611</v>
@@ -44409,7 +44495,7 @@
         <v>3.722</v>
       </c>
       <c r="V154" t="n">
-        <v>18205.90499999999</v>
+        <v>18205.905</v>
       </c>
       <c r="W154" t="n">
         <v>-11.997</v>

</xml_diff>

<commit_message>
Cap nhat ALM cac ma dang missing — Q3-2025 — 2026-09-17
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -32687,7 +32687,7 @@
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>2026-08-31T15:15:38+07:00</t>
+          <t>2026-09-17T17:29:41+07:00</t>
         </is>
       </c>
     </row>
@@ -34948,12 +34948,79 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>781937.368</v>
+      </c>
+      <c r="F46" t="n">
+        <v>68407.053</v>
+      </c>
+      <c r="G46" t="n">
+        <v>7763.322</v>
+      </c>
+      <c r="H46" t="n">
+        <v>487862.978</v>
+      </c>
+      <c r="I46" t="n">
+        <v>482446.82</v>
+      </c>
+      <c r="J46" t="n">
+        <v>98.89</v>
+      </c>
+      <c r="K46" t="n">
+        <v>182275.996</v>
+      </c>
+      <c r="L46" t="n">
+        <v>32.341</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="N46" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="U46" t="n">
+        <v>3.736</v>
+      </c>
+      <c r="V46" t="n">
+        <v>0</v>
+      </c>
+      <c r="W46" t="n">
+        <v>0</v>
+      </c>
+      <c r="X46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF46" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 3 năm 2025</t>
+        </is>
+      </c>
+      <c r="AG46" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20251030_-_HDB_-_BCTC_hop_nhat_Quy_3_nam_2025_1761869961.pdf</t>
         </is>
       </c>
       <c r="AH46" t="inlineStr">
         <is>
-          <t>2026-08-31T15:23:24+07:00</t>
+          <t>2026-09-17T17:31:12+07:00</t>
         </is>
       </c>
     </row>
@@ -38855,12 +38922,103 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>315161.711371066</v>
+      </c>
+      <c r="F88" t="n">
+        <v>32647.855006504</v>
+      </c>
+      <c r="G88" t="n">
+        <v>2424.219290094</v>
+      </c>
+      <c r="H88" t="n">
+        <v>155238.508114289</v>
+      </c>
+      <c r="I88" t="n">
+        <v>192730.756354787</v>
+      </c>
+      <c r="J88" t="n">
+        <v>124.151</v>
+      </c>
+      <c r="K88" t="n">
+        <v>55915.74639558799</v>
+      </c>
+      <c r="L88" t="n">
+        <v>-122022.499097568</v>
+      </c>
+      <c r="M88" t="n">
+        <v>-38.717</v>
+      </c>
+      <c r="N88" t="n">
+        <v>-51.884</v>
+      </c>
+      <c r="O88" t="n">
+        <v>-51.884</v>
+      </c>
+      <c r="P88" t="n">
+        <v>163519.653</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>60858.551</v>
+      </c>
+      <c r="R88" t="n">
+        <v>268.688</v>
+      </c>
+      <c r="S88" t="n">
+        <v>95.196</v>
+      </c>
+      <c r="T88" t="n">
+        <v>105.046</v>
+      </c>
+      <c r="U88" t="n">
+        <v>3.602</v>
+      </c>
+      <c r="V88" t="n">
+        <v>-163515.422343776</v>
+      </c>
+      <c r="W88" t="n">
+        <v>-38.716</v>
+      </c>
+      <c r="X88" t="n">
+        <v>-51.883</v>
+      </c>
+      <c r="Y88" t="n">
+        <v>-51.883</v>
+      </c>
+      <c r="Z88" t="n">
+        <v>141033.646</v>
+      </c>
+      <c r="AA88" t="n">
+        <v>230768.26</v>
+      </c>
+      <c r="AB88" t="n">
+        <v>61.115</v>
+      </c>
+      <c r="AC88" t="n">
+        <v>-1515</v>
+      </c>
+      <c r="AD88" t="n">
+        <v>-62.494</v>
+      </c>
+      <c r="AE88" t="n">
+        <v>-4.64</v>
+      </c>
+      <c r="AF88" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 3 năm 2025</t>
+        </is>
+      </c>
+      <c r="AG88" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20251028_-_OCB_-_BCTC_hop_nhat_Quy_3_2025_1761822426.pdf</t>
         </is>
       </c>
       <c r="AH88" t="inlineStr">
         <is>
-          <t>2026-08-31T15:37:44+07:00</t>
+          <t>2026-09-17T17:33:01+07:00</t>
         </is>
       </c>
     </row>
@@ -40314,7 +40472,7 @@
       </c>
       <c r="AH106" t="inlineStr">
         <is>
-          <t>2026-08-31T15:42:17+07:00</t>
+          <t>2026-09-17T17:34:13+07:00</t>
         </is>
       </c>
     </row>
@@ -42510,12 +42668,103 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>451893.195</v>
+      </c>
+      <c r="F130" t="n">
+        <v>39993.24</v>
+      </c>
+      <c r="G130" t="n">
+        <v>3237.619</v>
+      </c>
+      <c r="H130" t="n">
+        <v>260245.786</v>
+      </c>
+      <c r="I130" t="n">
+        <v>292020.111</v>
+      </c>
+      <c r="J130" t="n">
+        <v>112.209</v>
+      </c>
+      <c r="K130" t="n">
+        <v>87563.264</v>
+      </c>
+      <c r="L130" t="n">
+        <v>-224607.003</v>
+      </c>
+      <c r="M130" t="n">
+        <v>-49.704</v>
+      </c>
+      <c r="N130" t="n">
+        <v>-53.901</v>
+      </c>
+      <c r="O130" t="n">
+        <v>-36.315</v>
+      </c>
+      <c r="P130" t="n">
+        <v>411899.955</v>
+      </c>
+      <c r="Q130" t="n">
+        <v>208233.938</v>
+      </c>
+      <c r="R130" t="n">
+        <v>197.806</v>
+      </c>
+      <c r="S130" t="n">
+        <v>217.528</v>
+      </c>
+      <c r="T130" t="n">
+        <v>45.971</v>
+      </c>
+      <c r="U130" t="n">
+        <v>3.365</v>
+      </c>
+      <c r="V130" t="n">
+        <v>-263132.046</v>
+      </c>
+      <c r="W130" t="n">
+        <v>-2.247</v>
+      </c>
+      <c r="X130" t="n">
+        <v>-6.445</v>
+      </c>
+      <c r="Y130" t="n">
+        <v>-58.229</v>
+      </c>
+      <c r="Z130" t="n">
+        <v>909690.326</v>
+      </c>
+      <c r="AA130" t="n">
+        <v>608057.379</v>
+      </c>
+      <c r="AB130" t="n">
+        <v>149.606</v>
+      </c>
+      <c r="AC130" t="n">
+        <v>-542</v>
+      </c>
+      <c r="AD130" t="n">
+        <v>-16.741</v>
+      </c>
+      <c r="AE130" t="n">
+        <v>-1.355</v>
+      </c>
+      <c r="AF130" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 3 năm 2025</t>
+        </is>
+      </c>
+      <c r="AG130" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20251030_-_TPB_-_Bao_cao_tai_chinh_hop_nhat_Q3.2025_signed_1761832307.pdf</t>
         </is>
       </c>
       <c r="AH130" t="inlineStr">
         <is>
-          <t>2026-08-31T15:53:04+07:00</t>
+          <t>2026-09-17T17:36:04+07:00</t>
         </is>
       </c>
     </row>
@@ -42924,7 +43173,7 @@
       </c>
       <c r="AH136" t="inlineStr">
         <is>
-          <t>2026-08-31T15:57:08+07:00</t>
+          <t>2026-09-17T17:39:50+07:00</t>
         </is>
       </c>
     </row>
@@ -43943,12 +44192,103 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>2378185.628</v>
+      </c>
+      <c r="F148" t="n">
+        <v>222791.545</v>
+      </c>
+      <c r="G148" t="n">
+        <v>14657.24</v>
+      </c>
+      <c r="H148" t="n">
+        <v>1611966.698</v>
+      </c>
+      <c r="I148" t="n">
+        <v>1595933.982</v>
+      </c>
+      <c r="J148" t="n">
+        <v>99.005</v>
+      </c>
+      <c r="K148" t="n">
+        <v>567345.417</v>
+      </c>
+      <c r="L148" t="n">
+        <v>-505610.893</v>
+      </c>
+      <c r="M148" t="n">
+        <v>-21.26</v>
+      </c>
+      <c r="N148" t="n">
+        <v>-15.851</v>
+      </c>
+      <c r="O148" t="n">
+        <v>-15.224</v>
+      </c>
+      <c r="P148" t="n">
+        <v>2136177.852</v>
+      </c>
+      <c r="Q148" t="n">
+        <v>633448.997</v>
+      </c>
+      <c r="R148" t="n">
+        <v>337.23</v>
+      </c>
+      <c r="S148" t="n">
+        <v>37.415</v>
+      </c>
+      <c r="T148" t="n">
+        <v>267.269</v>
+      </c>
+      <c r="U148" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="V148" t="n">
+        <v>-50506.96400000001</v>
+      </c>
+      <c r="W148" t="n">
+        <v>-16.271</v>
+      </c>
+      <c r="X148" t="n">
+        <v>-5.369</v>
+      </c>
+      <c r="Y148" t="n">
+        <v>-2.124</v>
+      </c>
+      <c r="Z148" t="n">
+        <v>523906.365</v>
+      </c>
+      <c r="AA148" t="n">
+        <v>318283.844</v>
+      </c>
+      <c r="AB148" t="n">
+        <v>164.604</v>
+      </c>
+      <c r="AC148" t="n">
+        <v>-656</v>
+      </c>
+      <c r="AD148" t="n">
+        <v>-4.476</v>
+      </c>
+      <c r="AE148" t="n">
+        <v>-0.294</v>
+      </c>
+      <c r="AF148" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 3 năm 2025</t>
+        </is>
+      </c>
+      <c r="AG148" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20251030_-_VCB_-_CBTT_BCTC_Hop_nhat_Q3.2025_1761883208.pdf</t>
         </is>
       </c>
       <c r="AH148" t="inlineStr">
         <is>
-          <t>2026-08-31T16:01:32+07:00</t>
+          <t>2026-09-17T17:41:27+07:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cap nhat ALM cac ma dang missing — Q1-2026 — 2026-09-17
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -36477,12 +36477,94 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>580859.917</v>
+      </c>
+      <c r="F60" t="n">
+        <v>49471.665</v>
+      </c>
+      <c r="G60" t="n">
+        <v>3878.245</v>
+      </c>
+      <c r="H60" t="n">
+        <v>345760.324</v>
+      </c>
+      <c r="I60" t="n">
+        <v>397873.229</v>
+      </c>
+      <c r="J60" t="n">
+        <v>115.072</v>
+      </c>
+      <c r="K60" t="n">
+        <v>109738.331</v>
+      </c>
+      <c r="L60" t="n">
+        <v>-331251.879</v>
+      </c>
+      <c r="M60" t="n">
+        <v>-57.028</v>
+      </c>
+      <c r="N60" t="n">
+        <v>-55.582</v>
+      </c>
+      <c r="O60" t="n">
+        <v>-55.571</v>
+      </c>
+      <c r="P60" t="n">
+        <v>347607.222</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>586084.463</v>
+      </c>
+      <c r="R60" t="n">
+        <v>59.31</v>
+      </c>
+      <c r="S60" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="T60" t="n">
+        <v>799.979</v>
+      </c>
+      <c r="U60" t="n">
+        <v>3.174</v>
+      </c>
+      <c r="V60" t="n">
+        <v>0</v>
+      </c>
+      <c r="W60" t="n">
+        <v>0</v>
+      </c>
+      <c r="X60" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF60" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="AG60" t="inlineStr">
+        <is>
+          <t>https://cdn.24hmoney.vn/upload/file/2026-2/2026-04-22/no-name-1776797412.pdf</t>
         </is>
       </c>
       <c r="AH60" t="inlineStr">
         <is>
-          <t>2026-09-17T09:43:14+07:00</t>
+          <t>2026-09-17T19:14:13+07:00</t>
         </is>
       </c>
     </row>
@@ -39443,12 +39525,103 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>344097.628063307</v>
+      </c>
+      <c r="F91" t="n">
+        <v>34900.70310944</v>
+      </c>
+      <c r="G91" t="n">
+        <v>2382.731946497</v>
+      </c>
+      <c r="H91" t="n">
+        <v>158683.19610787</v>
+      </c>
+      <c r="I91" t="n">
+        <v>200503.421569508</v>
+      </c>
+      <c r="J91" t="n">
+        <v>126.355</v>
+      </c>
+      <c r="K91" t="n">
+        <v>70288.959484693</v>
+      </c>
+      <c r="L91" t="n">
+        <v>1187.641439761</v>
+      </c>
+      <c r="M91" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="N91" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="P91" t="n">
+        <v>0.193</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>92.95</v>
+      </c>
+      <c r="R91" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="S91" t="n">
+        <v>37547.712</v>
+      </c>
+      <c r="T91" t="n">
+        <v>0.266</v>
+      </c>
+      <c r="U91" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="V91" t="n">
+        <v>-0.192697418</v>
+      </c>
+      <c r="W91" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X91" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Y91" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Z91" t="n">
+        <v>92.95</v>
+      </c>
+      <c r="AA91" t="n">
+        <v>0.224</v>
+      </c>
+      <c r="AB91" t="n">
+        <v>41547.537</v>
+      </c>
+      <c r="AC91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF91" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="AG91" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20260422_-_OCB_-_BCTC_hop_nhat_Quy_1_2026_1776854955.pdf</t>
         </is>
       </c>
       <c r="AH91" t="inlineStr">
         <is>
-          <t>2026-09-17T09:46:33+07:00</t>
+          <t>2026-09-17T19:15:32+07:00</t>
         </is>
       </c>
     </row>
@@ -40993,7 +41166,7 @@
       </c>
       <c r="AH109" t="inlineStr">
         <is>
-          <t>2026-09-17T09:48:13+07:00</t>
+          <t>2026-09-17T19:16:33+07:00</t>
         </is>
       </c>
     </row>
@@ -43347,12 +43520,103 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>527169.377</v>
+      </c>
+      <c r="F133" t="n">
+        <v>48034.318</v>
+      </c>
+      <c r="G133" t="n">
+        <v>3459.591</v>
+      </c>
+      <c r="H133" t="n">
+        <v>267038.156</v>
+      </c>
+      <c r="I133" t="n">
+        <v>312044.784</v>
+      </c>
+      <c r="J133" t="n">
+        <v>116.854</v>
+      </c>
+      <c r="K133" t="n">
+        <v>121977.888</v>
+      </c>
+      <c r="L133" t="n">
+        <v>861.6610000000001</v>
+      </c>
+      <c r="M133" t="n">
+        <v>0.163</v>
+      </c>
+      <c r="N133" t="n">
+        <v>0.174</v>
+      </c>
+      <c r="O133" t="n">
+        <v>0.348</v>
+      </c>
+      <c r="P133" t="n">
+        <v>68366.49800000001</v>
+      </c>
+      <c r="Q133" t="n">
+        <v>24031.185</v>
+      </c>
+      <c r="R133" t="n">
+        <v>284.491</v>
+      </c>
+      <c r="S133" t="n">
+        <v>201.128</v>
+      </c>
+      <c r="T133" t="n">
+        <v>49.719</v>
+      </c>
+      <c r="U133" t="n">
+        <v>4.568</v>
+      </c>
+      <c r="V133" t="n">
+        <v>22216.787</v>
+      </c>
+      <c r="W133" t="n">
+        <v>0</v>
+      </c>
+      <c r="X133" t="n">
+        <v>-0.915</v>
+      </c>
+      <c r="Y133" t="n">
+        <v>4.214</v>
+      </c>
+      <c r="Z133" t="n">
+        <v>201987.137</v>
+      </c>
+      <c r="AA133" t="n">
+        <v>63845.469</v>
+      </c>
+      <c r="AB133" t="n">
+        <v>316.369</v>
+      </c>
+      <c r="AC133" t="n">
+        <v>159</v>
+      </c>
+      <c r="AD133" t="n">
+        <v>4.596</v>
+      </c>
+      <c r="AE133" t="n">
+        <v>0.331</v>
+      </c>
+      <c r="AF133" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="AG133" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20260429_-_TPB_-_BCTC_hop_nhat_Quy_1_2026_signed_1777457982.pdf</t>
         </is>
       </c>
       <c r="AH133" t="inlineStr">
         <is>
-          <t>2026-09-17T09:59:43+07:00</t>
+          <t>2026-09-17T19:18:12+07:00</t>
         </is>
       </c>
     </row>
@@ -43776,7 +44040,7 @@
       </c>
       <c r="AH139" t="inlineStr">
         <is>
-          <t>2026-09-17T09:59:50+07:00</t>
+          <t>2026-09-17T19:18:18+07:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bank ALM: nhap thu cong VAB 2026-Q1 tu anh chup BCTC that
VAB in cot "Qua han duoi 3 thang" TRUOC "Qua han tren 3 thang" - dao nguoc thu
tu chuan (LIQUIDITY_BUCKETS gia dinh tren_3t truoc) - da doi cho lai khi nhap
tay. Don vi da xac nhan la Trieu dong that (khong phai VND thuc du bang co in
"VNĐ" lap lai - xem phat hien va fix ebf0ffc) qua doi chieu voi
quarterly_balance_sheet doc lap tu Vietcap (142.390 ty, khop voi 143.740 ty
suy tu bang gap KHONG can quy doi them). Da doi chieu 2 chieu truoc khi nhap.

Luu y con lai (chua sua, muc do anh huong nho): thu tu cot "qua han duoi/tren
3 thang" khac nhau giua cac ngan hang co the anh huong nhe do chinh xac cua
OCR tu dong trich 2 bucket qua han dau tien neu chay lai qua che do OCR that
(khong anh huong du lieu nhap tay nay).
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30918,7 +30918,7 @@
         <v>4.068</v>
       </c>
       <c r="V4" t="n">
-        <v>8183.362999999996</v>
+        <v>8183.362999999999</v>
       </c>
       <c r="W4" t="n">
         <v>-7.633</v>
@@ -31007,7 +31007,7 @@
         <v>3.572</v>
       </c>
       <c r="V5" t="n">
-        <v>-2072.081999999995</v>
+        <v>-2072.081999999999</v>
       </c>
       <c r="W5" t="n">
         <v>-6.467</v>
@@ -31111,7 +31111,7 @@
         <v>4.395</v>
       </c>
       <c r="V6" t="n">
-        <v>-5551.592999999999</v>
+        <v>-5551.593000000001</v>
       </c>
       <c r="W6" t="n">
         <v>0.38</v>
@@ -31408,7 +31408,7 @@
         <v>2.424</v>
       </c>
       <c r="V9" t="n">
-        <v>85041.65799999997</v>
+        <v>85041.658</v>
       </c>
       <c r="W9" t="n">
         <v>-9.567</v>
@@ -33050,7 +33050,7 @@
         <v>2.564</v>
       </c>
       <c r="V26" t="n">
-        <v>-2093.93</v>
+        <v>-2093.930000000001</v>
       </c>
       <c r="W26" t="n">
         <v>0</v>
@@ -34149,7 +34149,7 @@
         <v>584740.964</v>
       </c>
       <c r="L37" t="n">
-        <v>57219.16100000001</v>
+        <v>57219.161</v>
       </c>
       <c r="M37" t="n">
         <v>1.932</v>
@@ -34461,7 +34461,7 @@
         <v>2.439</v>
       </c>
       <c r="V40" t="n">
-        <v>-6843.675999999999</v>
+        <v>-6843.676</v>
       </c>
       <c r="W40" t="n">
         <v>-9.135999999999999</v>
@@ -34639,7 +34639,7 @@
         <v>42408.00799999999</v>
       </c>
       <c r="L42" t="n">
-        <v>2554.764000000001</v>
+        <v>2554.764</v>
       </c>
       <c r="M42" t="n">
         <v>0.946</v>
@@ -35385,7 +35385,7 @@
         <v>3.011</v>
       </c>
       <c r="V49" t="n">
-        <v>1097.082999999999</v>
+        <v>1097.083000000001</v>
       </c>
       <c r="W49" t="n">
         <v>3.244</v>
@@ -37304,7 +37304,7 @@
         <v>53049.641</v>
       </c>
       <c r="L68" t="n">
-        <v>-71627.23300000001</v>
+        <v>-71627.23299999999</v>
       </c>
       <c r="M68" t="n">
         <v>-22.759</v>
@@ -37646,7 +37646,7 @@
         <v>4.335</v>
       </c>
       <c r="V71" t="n">
-        <v>-36336.33499999999</v>
+        <v>-36336.335</v>
       </c>
       <c r="W71" t="n">
         <v>7.502</v>
@@ -37928,7 +37928,7 @@
         <v>3.04</v>
       </c>
       <c r="V74" t="n">
-        <v>1044.137999999999</v>
+        <v>1044.137999999998</v>
       </c>
       <c r="W74" t="n">
         <v>-0.302</v>
@@ -38032,7 +38032,7 @@
         <v>4.485</v>
       </c>
       <c r="V75" t="n">
-        <v>-7342.066000000003</v>
+        <v>-7342.066000000001</v>
       </c>
       <c r="W75" t="n">
         <v>1.12</v>
@@ -38819,7 +38819,7 @@
         <v>3.06</v>
       </c>
       <c r="V83" t="n">
-        <v>44447.072</v>
+        <v>44447.07199999999</v>
       </c>
       <c r="W83" t="n">
         <v>41.067</v>
@@ -39415,7 +39415,7 @@
         <v>57104.9273618</v>
       </c>
       <c r="L89" t="n">
-        <v>-8354.105685278017</v>
+        <v>-8354.105685278011</v>
       </c>
       <c r="M89" t="n">
         <v>-2.587</v>
@@ -40079,7 +40079,7 @@
         <v>6.429</v>
       </c>
       <c r="V96" t="n">
-        <v>-448.712</v>
+        <v>-448.7119999999998</v>
       </c>
       <c r="W96" t="n">
         <v>-8.398</v>
@@ -40361,7 +40361,7 @@
         <v>3.682</v>
       </c>
       <c r="V99" t="n">
-        <v>-8415.234000000002</v>
+        <v>-8415.234</v>
       </c>
       <c r="W99" t="n">
         <v>-5.98</v>
@@ -42835,7 +42835,7 @@
         <v>3.255</v>
       </c>
       <c r="V126" t="n">
-        <v>-95355.82799999998</v>
+        <v>-95355.82799999999</v>
       </c>
       <c r="W126" t="n">
         <v>-8.385</v>
@@ -42939,7 +42939,7 @@
         <v>3.105</v>
       </c>
       <c r="V127" t="n">
-        <v>31803.23300000001</v>
+        <v>31803.233</v>
       </c>
       <c r="W127" t="n">
         <v>4.369</v>
@@ -43043,7 +43043,7 @@
         <v>2.784</v>
       </c>
       <c r="V128" t="n">
-        <v>49624.19500000001</v>
+        <v>49624.19499999999</v>
       </c>
       <c r="W128" t="n">
         <v>9.231999999999999</v>
@@ -43147,7 +43147,7 @@
         <v>2.296</v>
       </c>
       <c r="V129" t="n">
-        <v>47597.061</v>
+        <v>47597.06099999999</v>
       </c>
       <c r="W129" t="n">
         <v>12.611</v>
@@ -44035,12 +44035,98 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>142390.241306315</v>
+      </c>
+      <c r="F139" t="n">
+        <v>10569.944213453</v>
+      </c>
+      <c r="G139" t="n">
+        <v>675.525473695</v>
+      </c>
+      <c r="H139" t="n">
+        <v>102351.029371344</v>
+      </c>
+      <c r="I139" t="n">
+        <v>89679.977935756</v>
+      </c>
+      <c r="J139" t="n">
+        <v>87.62</v>
+      </c>
+      <c r="K139" t="n">
+        <v>19802.319642618</v>
+      </c>
+      <c r="L139" t="n">
+        <v>21287.514</v>
+      </c>
+      <c r="M139" t="n">
+        <v>14.95</v>
+      </c>
+      <c r="N139" t="n">
+        <v>9.039</v>
+      </c>
+      <c r="O139" t="n">
+        <v>-8.877000000000001</v>
+      </c>
+      <c r="P139" t="n">
+        <v>127900.126</v>
+      </c>
+      <c r="Q139" t="n">
+        <v>28479.752</v>
+      </c>
+      <c r="R139" t="n">
+        <v>449.091</v>
+      </c>
+      <c r="S139" t="n">
+        <v>50.879</v>
+      </c>
+      <c r="T139" t="n">
+        <v>196.546</v>
+      </c>
+      <c r="U139" t="n">
+        <v>1.935</v>
+      </c>
+      <c r="V139" t="n">
+        <v>3955.387000000001</v>
+      </c>
+      <c r="W139" t="n">
+        <v>-2.566</v>
+      </c>
+      <c r="X139" t="n">
+        <v>7.933</v>
+      </c>
+      <c r="Y139" t="n">
+        <v>2.778</v>
+      </c>
+      <c r="Z139" t="n">
+        <v>131635.815</v>
+      </c>
+      <c r="AA139" t="n">
+        <v>129515.728</v>
+      </c>
+      <c r="AB139" t="n">
+        <v>101.637</v>
+      </c>
+      <c r="AC139" t="n">
+        <v>89</v>
+      </c>
+      <c r="AD139" t="n">
+        <v>13.175</v>
+      </c>
+      <c r="AE139" t="n">
+        <v>0.842</v>
+      </c>
+      <c r="AF139" t="inlineStr">
+        <is>
+          <t>Nhap thu cong tu anh chup BCTC that (VAB thuyet minh BCTC Quy 1 2026, cot 'qua han duoi/tren 3 thang' dao nguoc thu tu so voi chuan nen da doi lai khi nhap, don vi da xac nhan la Trieu dong that qua doi chieu Vietcap)</t>
         </is>
       </c>
       <c r="AH139" t="inlineStr">
         <is>
-          <t>2026-09-18T08:14:13+07:00</t>
+          <t>2026-09-18T08:32:03+07:00</t>
         </is>
       </c>
     </row>
@@ -45576,7 +45662,7 @@
         <v>3.722</v>
       </c>
       <c r="V155" t="n">
-        <v>18205.90499999999</v>
+        <v>18205.905</v>
       </c>
       <c r="W155" t="n">
         <v>-11.997</v>

</xml_diff>

<commit_message>
Cap nhat ALM VAB — Q3-2025 — 2026-09-18
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30918,7 +30918,7 @@
         <v>4.068</v>
       </c>
       <c r="V4" t="n">
-        <v>8183.362999999999</v>
+        <v>8183.362999999996</v>
       </c>
       <c r="W4" t="n">
         <v>-7.633</v>
@@ -31007,7 +31007,7 @@
         <v>3.572</v>
       </c>
       <c r="V5" t="n">
-        <v>-2072.081999999999</v>
+        <v>-2072.081999999995</v>
       </c>
       <c r="W5" t="n">
         <v>-6.467</v>
@@ -31111,7 +31111,7 @@
         <v>4.395</v>
       </c>
       <c r="V6" t="n">
-        <v>-5551.593000000001</v>
+        <v>-5551.592999999999</v>
       </c>
       <c r="W6" t="n">
         <v>0.38</v>
@@ -31408,7 +31408,7 @@
         <v>2.424</v>
       </c>
       <c r="V9" t="n">
-        <v>85041.658</v>
+        <v>85041.65799999997</v>
       </c>
       <c r="W9" t="n">
         <v>-9.567</v>
@@ -33050,7 +33050,7 @@
         <v>2.564</v>
       </c>
       <c r="V26" t="n">
-        <v>-2093.930000000001</v>
+        <v>-2093.93</v>
       </c>
       <c r="W26" t="n">
         <v>0</v>
@@ -34149,7 +34149,7 @@
         <v>584740.964</v>
       </c>
       <c r="L37" t="n">
-        <v>57219.161</v>
+        <v>57219.16100000001</v>
       </c>
       <c r="M37" t="n">
         <v>1.932</v>
@@ -34461,7 +34461,7 @@
         <v>2.439</v>
       </c>
       <c r="V40" t="n">
-        <v>-6843.676</v>
+        <v>-6843.675999999999</v>
       </c>
       <c r="W40" t="n">
         <v>-9.135999999999999</v>
@@ -34639,7 +34639,7 @@
         <v>42408.00799999999</v>
       </c>
       <c r="L42" t="n">
-        <v>2554.764</v>
+        <v>2554.764000000001</v>
       </c>
       <c r="M42" t="n">
         <v>0.946</v>
@@ -35385,7 +35385,7 @@
         <v>3.011</v>
       </c>
       <c r="V49" t="n">
-        <v>1097.083000000001</v>
+        <v>1097.082999999999</v>
       </c>
       <c r="W49" t="n">
         <v>3.244</v>
@@ -37304,7 +37304,7 @@
         <v>53049.641</v>
       </c>
       <c r="L68" t="n">
-        <v>-71627.23299999999</v>
+        <v>-71627.23300000001</v>
       </c>
       <c r="M68" t="n">
         <v>-22.759</v>
@@ -37646,7 +37646,7 @@
         <v>4.335</v>
       </c>
       <c r="V71" t="n">
-        <v>-36336.335</v>
+        <v>-36336.33499999999</v>
       </c>
       <c r="W71" t="n">
         <v>7.502</v>
@@ -37928,7 +37928,7 @@
         <v>3.04</v>
       </c>
       <c r="V74" t="n">
-        <v>1044.137999999998</v>
+        <v>1044.137999999999</v>
       </c>
       <c r="W74" t="n">
         <v>-0.302</v>
@@ -38032,7 +38032,7 @@
         <v>4.485</v>
       </c>
       <c r="V75" t="n">
-        <v>-7342.066000000001</v>
+        <v>-7342.066000000003</v>
       </c>
       <c r="W75" t="n">
         <v>1.12</v>
@@ -38819,7 +38819,7 @@
         <v>3.06</v>
       </c>
       <c r="V83" t="n">
-        <v>44447.07199999999</v>
+        <v>44447.072</v>
       </c>
       <c r="W83" t="n">
         <v>41.067</v>
@@ -39415,7 +39415,7 @@
         <v>57104.9273618</v>
       </c>
       <c r="L89" t="n">
-        <v>-8354.105685278011</v>
+        <v>-8354.105685278017</v>
       </c>
       <c r="M89" t="n">
         <v>-2.587</v>
@@ -40079,7 +40079,7 @@
         <v>6.429</v>
       </c>
       <c r="V96" t="n">
-        <v>-448.7119999999998</v>
+        <v>-448.712</v>
       </c>
       <c r="W96" t="n">
         <v>-8.398</v>
@@ -40361,7 +40361,7 @@
         <v>3.682</v>
       </c>
       <c r="V99" t="n">
-        <v>-8415.234</v>
+        <v>-8415.234000000002</v>
       </c>
       <c r="W99" t="n">
         <v>-5.98</v>
@@ -42835,7 +42835,7 @@
         <v>3.255</v>
       </c>
       <c r="V126" t="n">
-        <v>-95355.82799999999</v>
+        <v>-95355.82799999998</v>
       </c>
       <c r="W126" t="n">
         <v>-8.385</v>
@@ -42939,7 +42939,7 @@
         <v>3.105</v>
       </c>
       <c r="V127" t="n">
-        <v>31803.233</v>
+        <v>31803.23300000001</v>
       </c>
       <c r="W127" t="n">
         <v>4.369</v>
@@ -43043,7 +43043,7 @@
         <v>2.784</v>
       </c>
       <c r="V128" t="n">
-        <v>49624.19499999999</v>
+        <v>49624.19500000001</v>
       </c>
       <c r="W128" t="n">
         <v>9.231999999999999</v>
@@ -43147,7 +43147,7 @@
         <v>2.296</v>
       </c>
       <c r="V129" t="n">
-        <v>47597.06099999999</v>
+        <v>47597.061</v>
       </c>
       <c r="W129" t="n">
         <v>12.611</v>
@@ -43909,12 +43909,88 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>134613.747271322</v>
+      </c>
+      <c r="F137" t="n">
+        <v>9690.784798859</v>
+      </c>
+      <c r="G137" t="n">
+        <v>638.68127616</v>
+      </c>
+      <c r="H137" t="n">
+        <v>97984.432309576</v>
+      </c>
+      <c r="I137" t="n">
+        <v>85811.150481169</v>
+      </c>
+      <c r="J137" t="n">
+        <v>87.57599999999999</v>
+      </c>
+      <c r="K137" t="n">
+        <v>20755.174731968</v>
+      </c>
+      <c r="L137" t="n">
+        <v>0</v>
+      </c>
+      <c r="M137" t="n">
+        <v>0</v>
+      </c>
+      <c r="N137" t="n">
+        <v>0</v>
+      </c>
+      <c r="O137" t="n">
+        <v>0</v>
+      </c>
+      <c r="U137" t="n">
+        <v>2.118</v>
+      </c>
+      <c r="V137" t="n">
+        <v>5430.341</v>
+      </c>
+      <c r="W137" t="n">
+        <v>-1.568</v>
+      </c>
+      <c r="X137" t="n">
+        <v>10.425</v>
+      </c>
+      <c r="Y137" t="n">
+        <v>4.034</v>
+      </c>
+      <c r="Z137" t="n">
+        <v>221001.348</v>
+      </c>
+      <c r="AA137" t="n">
+        <v>221087.326</v>
+      </c>
+      <c r="AB137" t="n">
+        <v>99.961</v>
+      </c>
+      <c r="AC137" t="n">
+        <v>93</v>
+      </c>
+      <c r="AD137" t="n">
+        <v>14.561</v>
+      </c>
+      <c r="AE137" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AF137" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 3 năm 2025</t>
+        </is>
+      </c>
+      <c r="AG137" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20251017_-_VAB_-_BCTC_HN_Q3.2025_1761126486.pdf</t>
         </is>
       </c>
       <c r="AH137" t="inlineStr">
         <is>
-          <t>2026-09-17T18:14:21+07:00</t>
+          <t>2026-09-18T08:37:05+07:00</t>
         </is>
       </c>
     </row>
@@ -45662,7 +45738,7 @@
         <v>3.722</v>
       </c>
       <c r="V155" t="n">
-        <v>18205.905</v>
+        <v>18205.90499999999</v>
       </c>
       <c r="W155" t="n">
         <v>-11.997</v>

</xml_diff>

<commit_message>
Cap nhat ALM bid — Q3-2025 — 2026-09-18
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -32682,12 +32682,97 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>3071970.196</v>
+      </c>
+      <c r="F22" t="n">
+        <v>167986.701</v>
+      </c>
+      <c r="G22" t="n">
+        <v>15172.618</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2087181.421</v>
+      </c>
+      <c r="I22" t="n">
+        <v>2197470.752</v>
+      </c>
+      <c r="J22" t="n">
+        <v>105.284</v>
+      </c>
+      <c r="K22" t="n">
+        <v>512310.713</v>
+      </c>
+      <c r="L22" t="n">
+        <v>20511.126</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.668</v>
+      </c>
+      <c r="N22" t="n">
+        <v>2.237</v>
+      </c>
+      <c r="O22" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="P22" t="n">
+        <v>7048.125</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" t="n">
+        <v>2.455</v>
+      </c>
+      <c r="V22" t="n">
+        <v>459217.92</v>
+      </c>
+      <c r="W22" t="n">
+        <v>7.618</v>
+      </c>
+      <c r="X22" t="n">
+        <v>23.135</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>14.949</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>1186171.693</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>441729.583</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>268.529</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>4337</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>28.584</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>2.582</v>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 3 năm 2025</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20251030_-_BID_-_CBTT_BCTC_HN_giua_nien_do_QIII_1761898492.pdf</t>
         </is>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>2026-09-17T18:09:51+07:00</t>
+          <t>2026-09-18T08:44:10+07:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cap nhat ALM cac ma dang missing — Q1-2024 — 2026-09-18
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALM_NganHang_RawBuckets" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ALM_NganHang_RawBuckets" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30963,7 +30963,7 @@
         <v>2.644</v>
       </c>
       <c r="AI2" t="n">
-        <v>5142.782000000002</v>
+        <v>5142.781999999998</v>
       </c>
       <c r="AJ2" t="n">
         <v>-6.842</v>
@@ -31124,7 +31124,7 @@
         <v>2.349</v>
       </c>
       <c r="AI3" t="n">
-        <v>6180.512000000001</v>
+        <v>6180.511999999999</v>
       </c>
       <c r="AJ3" t="n">
         <v>-6.22</v>
@@ -31529,7 +31529,7 @@
         <v>2.034</v>
       </c>
       <c r="AI6" t="n">
-        <v>8183.362999999999</v>
+        <v>8183.362999999996</v>
       </c>
       <c r="AJ6" t="n">
         <v>-7.633</v>
@@ -31651,7 +31651,7 @@
         <v>1.786</v>
       </c>
       <c r="AI7" t="n">
-        <v>-2072.081999999999</v>
+        <v>-2072.081999999995</v>
       </c>
       <c r="AJ7" t="n">
         <v>-6.467</v>
@@ -31803,7 +31803,7 @@
         <v>2.198</v>
       </c>
       <c r="AI8" t="n">
-        <v>-5551.593000000001</v>
+        <v>-5551.592999999999</v>
       </c>
       <c r="AJ8" t="n">
         <v>0.38</v>
@@ -32077,7 +32077,7 @@
         <v>1.383</v>
       </c>
       <c r="AI10" t="n">
-        <v>72159.24699999997</v>
+        <v>72159.24699999994</v>
       </c>
       <c r="AJ10" t="n">
         <v>-11.405</v>
@@ -32238,7 +32238,7 @@
         <v>1.248</v>
       </c>
       <c r="AI11" t="n">
-        <v>75182.47699999998</v>
+        <v>75182.47699999997</v>
       </c>
       <c r="AJ11" t="n">
         <v>-9.868</v>
@@ -32551,7 +32551,7 @@
         <v>1.212</v>
       </c>
       <c r="AI13" t="n">
-        <v>85041.658</v>
+        <v>85041.65799999997</v>
       </c>
       <c r="AJ13" t="n">
         <v>-9.567</v>
@@ -34664,7 +34664,7 @@
         <v>0.912</v>
       </c>
       <c r="AI27" t="n">
-        <v>482308.417</v>
+        <v>482308.4170000001</v>
       </c>
       <c r="AJ27" t="n">
         <v>12.989</v>
@@ -35994,7 +35994,7 @@
         <v>1.282</v>
       </c>
       <c r="AI36" t="n">
-        <v>-2093.930000000001</v>
+        <v>-2093.93</v>
       </c>
       <c r="AJ36" t="n">
         <v>0</v>
@@ -37895,7 +37895,7 @@
         <v>584740.964</v>
       </c>
       <c r="O49" t="n">
-        <v>57219.161</v>
+        <v>57219.16100000001</v>
       </c>
       <c r="P49" t="n">
         <v>1.932</v>
@@ -38169,7 +38169,7 @@
         <v>1.207</v>
       </c>
       <c r="AI51" t="n">
-        <v>536.0379999999996</v>
+        <v>536.0379999999986</v>
       </c>
       <c r="AJ51" t="n">
         <v>-8.407999999999999</v>
@@ -38595,7 +38595,7 @@
         <v>1.219</v>
       </c>
       <c r="AI54" t="n">
-        <v>-6843.676</v>
+        <v>-6843.675999999999</v>
       </c>
       <c r="AJ54" t="n">
         <v>-9.135999999999999</v>
@@ -38836,7 +38836,7 @@
         <v>42408.00799999999</v>
       </c>
       <c r="O56" t="n">
-        <v>2554.764</v>
+        <v>2554.764000000001</v>
       </c>
       <c r="P56" t="n">
         <v>0.946</v>
@@ -39128,7 +39128,7 @@
         <v>113076.542</v>
       </c>
       <c r="O58" t="n">
-        <v>89209.497</v>
+        <v>89209.49699999999</v>
       </c>
       <c r="P58" t="n">
         <v>14.805</v>
@@ -40180,7 +40180,7 @@
         <v>1.506</v>
       </c>
       <c r="AI65" t="n">
-        <v>1097.083000000001</v>
+        <v>1097.082999999999</v>
       </c>
       <c r="AJ65" t="n">
         <v>3.244</v>
@@ -42901,7 +42901,7 @@
         <v>0.909</v>
       </c>
       <c r="AI83" t="n">
-        <v>20403.41100000001</v>
+        <v>20403.411</v>
       </c>
       <c r="AJ83" t="n">
         <v>-10.621</v>
@@ -43843,7 +43843,7 @@
       </c>
       <c r="BL90" t="inlineStr">
         <is>
-          <t>2026-09-18T11:56:55+07:00</t>
+          <t>2026-09-18T16:44:46+07:00</t>
         </is>
       </c>
     </row>
@@ -44031,7 +44031,7 @@
         <v>53049.641</v>
       </c>
       <c r="O92" t="n">
-        <v>-71627.23299999999</v>
+        <v>-71627.23300000001</v>
       </c>
       <c r="P92" t="n">
         <v>-22.759</v>
@@ -44532,7 +44532,7 @@
         <v>2.167</v>
       </c>
       <c r="AI95" t="n">
-        <v>-36336.335</v>
+        <v>-36336.33499999999</v>
       </c>
       <c r="AJ95" t="n">
         <v>7.502</v>
@@ -44937,7 +44937,7 @@
         <v>1.218</v>
       </c>
       <c r="AI98" t="n">
-        <v>9206.203</v>
+        <v>9206.203000000001</v>
       </c>
       <c r="AJ98" t="n">
         <v>-4.209</v>
@@ -45229,7 +45229,7 @@
         <v>1.52</v>
       </c>
       <c r="AI100" t="n">
-        <v>1044.137999999998</v>
+        <v>1044.137999999999</v>
       </c>
       <c r="AJ100" t="n">
         <v>-0.302</v>
@@ -45381,7 +45381,7 @@
         <v>2.243</v>
       </c>
       <c r="AI101" t="n">
-        <v>-7342.066000000001</v>
+        <v>-7342.066000000003</v>
       </c>
       <c r="AJ101" t="n">
         <v>1.12</v>
@@ -46040,7 +46040,7 @@
       </c>
       <c r="BL106" t="inlineStr">
         <is>
-          <t>2026-09-18T12:00:15+07:00</t>
+          <t>2026-09-18T16:46:20+07:00</t>
         </is>
       </c>
     </row>
@@ -46097,7 +46097,7 @@
         <v>10333.757</v>
       </c>
       <c r="O107" t="n">
-        <v>4585.813</v>
+        <v>4585.812999999998</v>
       </c>
       <c r="P107" t="n">
         <v>4.439</v>
@@ -46684,7 +46684,7 @@
         <v>1.53</v>
       </c>
       <c r="AI111" t="n">
-        <v>44447.07199999999</v>
+        <v>44447.072</v>
       </c>
       <c r="AJ111" t="n">
         <v>41.067</v>
@@ -47053,7 +47053,7 @@
         <v>43767.119108461</v>
       </c>
       <c r="O114" t="n">
-        <v>45040.48364739501</v>
+        <v>45040.483647395</v>
       </c>
       <c r="P114" t="n">
         <v>19.006</v>
@@ -47104,7 +47104,7 @@
         <v>1.727</v>
       </c>
       <c r="AI114" t="n">
-        <v>73880.39491509201</v>
+        <v>73880.39491509199</v>
       </c>
       <c r="AJ114" t="n">
         <v>13.551</v>
@@ -47848,7 +47848,7 @@
         <v>57104.9273618</v>
       </c>
       <c r="O119" t="n">
-        <v>-8354.105685278011</v>
+        <v>-8354.105685278017</v>
       </c>
       <c r="P119" t="n">
         <v>-2.587</v>
@@ -48433,7 +48433,7 @@
       </c>
       <c r="BL123" t="inlineStr">
         <is>
-          <t>2026-09-18T12:03:53+07:00</t>
+          <t>2026-09-18T16:47:58+07:00</t>
         </is>
       </c>
     </row>
@@ -49107,7 +49107,7 @@
         <v>3.214</v>
       </c>
       <c r="AI128" t="n">
-        <v>-448.7119999999998</v>
+        <v>-448.712</v>
       </c>
       <c r="AJ128" t="n">
         <v>-8.398</v>
@@ -49462,7 +49462,7 @@
       </c>
       <c r="BL131" t="inlineStr">
         <is>
-          <t>2026-09-18T12:05:01+07:00</t>
+          <t>2026-09-18T16:49:11+07:00</t>
         </is>
       </c>
     </row>
@@ -49692,7 +49692,7 @@
         <v>1.841</v>
       </c>
       <c r="AI133" t="n">
-        <v>-8415.234</v>
+        <v>-8415.234000000002</v>
       </c>
       <c r="AJ133" t="n">
         <v>-5.98</v>
@@ -50470,7 +50470,7 @@
       </c>
       <c r="BL139" t="inlineStr">
         <is>
-          <t>2026-09-18T12:05:48+07:00</t>
+          <t>2026-09-18T16:49:58+07:00</t>
         </is>
       </c>
     </row>
@@ -50527,7 +50527,7 @@
         <v>110803.352</v>
       </c>
       <c r="O140" t="n">
-        <v>84929.84099999999</v>
+        <v>84929.841</v>
       </c>
       <c r="P140" t="n">
         <v>12.871</v>
@@ -54410,7 +54410,7 @@
         <v>1.628</v>
       </c>
       <c r="AI168" t="n">
-        <v>-95355.82799999999</v>
+        <v>-95355.82799999998</v>
       </c>
       <c r="AJ168" t="n">
         <v>-8.385</v>
@@ -54571,7 +54571,7 @@
         <v>1.553</v>
       </c>
       <c r="AI169" t="n">
-        <v>31803.233</v>
+        <v>31803.23300000001</v>
       </c>
       <c r="AJ169" t="n">
         <v>4.369</v>
@@ -54764,7 +54764,7 @@
         <v>1.392</v>
       </c>
       <c r="AI170" t="n">
-        <v>49624.19499999999</v>
+        <v>49624.19500000001</v>
       </c>
       <c r="AJ170" t="n">
         <v>9.231999999999999</v>
@@ -55253,7 +55253,7 @@
         <v>1.148</v>
       </c>
       <c r="AI173" t="n">
-        <v>47597.06099999999</v>
+        <v>47597.061</v>
       </c>
       <c r="AJ173" t="n">
         <v>12.611</v>
@@ -56158,7 +56158,7 @@
       </c>
       <c r="BL179" t="inlineStr">
         <is>
-          <t>2026-09-18T12:16:10+07:00</t>
+          <t>2026-09-18T16:52:58+07:00</t>
         </is>
       </c>
     </row>
@@ -56236,7 +56236,7 @@
         <v>0.951</v>
       </c>
       <c r="AI180" t="n">
-        <v>786.7630000000004</v>
+        <v>786.7630000000008</v>
       </c>
       <c r="AJ180" t="n">
         <v>0.008999999999999999</v>
@@ -57294,7 +57294,7 @@
       </c>
       <c r="BL187" t="inlineStr">
         <is>
-          <t>2026-09-18T12:17:37+07:00</t>
+          <t>2026-09-18T16:54:28+07:00</t>
         </is>
       </c>
     </row>
@@ -60095,7 +60095,7 @@
         <v>1.861</v>
       </c>
       <c r="AI207" t="n">
-        <v>18205.905</v>
+        <v>18205.90499999999</v>
       </c>
       <c r="AJ207" t="n">
         <v>-11.997</v>
@@ -72701,7 +72701,7 @@
       </c>
       <c r="CE90" t="inlineStr">
         <is>
-          <t>2026-09-18T11:56:55+07:00</t>
+          <t>2026-09-18T16:44:46+07:00</t>
         </is>
       </c>
     </row>
@@ -74586,7 +74586,7 @@
       </c>
       <c r="CE106" t="inlineStr">
         <is>
-          <t>2026-09-18T12:00:15+07:00</t>
+          <t>2026-09-18T16:46:20+07:00</t>
         </is>
       </c>
     </row>
@@ -76840,7 +76840,7 @@
       </c>
       <c r="CE123" t="inlineStr">
         <is>
-          <t>2026-09-18T12:03:53+07:00</t>
+          <t>2026-09-18T16:47:58+07:00</t>
         </is>
       </c>
     </row>
@@ -77702,7 +77702,7 @@
       </c>
       <c r="CE131" t="inlineStr">
         <is>
-          <t>2026-09-18T12:05:01+07:00</t>
+          <t>2026-09-18T16:49:11+07:00</t>
         </is>
       </c>
     </row>
@@ -78492,7 +78492,7 @@
       </c>
       <c r="CE139" t="inlineStr">
         <is>
-          <t>2026-09-18T12:05:48+07:00</t>
+          <t>2026-09-18T16:49:58+07:00</t>
         </is>
       </c>
     </row>
@@ -84009,7 +84009,7 @@
       </c>
       <c r="CE179" t="inlineStr">
         <is>
-          <t>2026-09-18T12:16:10+07:00</t>
+          <t>2026-09-18T16:52:58+07:00</t>
         </is>
       </c>
     </row>
@@ -85029,7 +85029,7 @@
       </c>
       <c r="CE187" t="inlineStr">
         <is>
-          <t>2026-09-18T12:17:37+07:00</t>
+          <t>2026-09-18T16:54:28+07:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Them bo OCR tu dong cho Rui ro tien te (FX position) + sua cot Trang thai tong hop
- _extract_fx_position()/_find_fx_currency_header() (bank_risk_notes.py): tu dong do trang
  "Rui ro tien te" (cot dong tien bien doi tuy ngan hang, khong co bucket co dinh nhu 2 bang
  lai suat/thanh khoan) va trich Tai san/No phai tra/Trang thai noi bang/ngoai bang/noi-ngoai
  bang theo tung dong tien - verify khop 7/7 voi anh chup that TCB Q1/2026 va BIDV Q3/2025
  (ke ca thu tu cot dao nguoc EUR truoc USD cua BIDV).
- Sua _strip_accents(): "Đ"/"đ" khong tu rut gon qua NFD (khong phai ky tu to hop) - can thay
  thu cong truoc, phat hien khi nhan "Do la My" khong khop duoc.
- Cot "Trang thai" (cot C) trong ca 2 sheet Excel gio la TONG HOP: missing neu 1 trong Lai
  suat/Thanh khoan con thieu (khong tinh Tien te - chua co OCR tu dong cho da so ma), giup
  kiem tra 1 cot duy nhat de biet co can cap nhat khong.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ALM_NganHang_RawBuckets" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALM_NganHang_RawBuckets" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30963,7 +30963,7 @@
         <v>2.644</v>
       </c>
       <c r="AI2" t="n">
-        <v>5142.781999999998</v>
+        <v>5142.782000000002</v>
       </c>
       <c r="AJ2" t="n">
         <v>-6.842</v>
@@ -31124,7 +31124,7 @@
         <v>2.349</v>
       </c>
       <c r="AI3" t="n">
-        <v>6180.511999999999</v>
+        <v>6180.512000000001</v>
       </c>
       <c r="AJ3" t="n">
         <v>-6.22</v>
@@ -31316,7 +31316,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -31529,7 +31529,7 @@
         <v>2.034</v>
       </c>
       <c r="AI6" t="n">
-        <v>8183.362999999996</v>
+        <v>8183.362999999999</v>
       </c>
       <c r="AJ6" t="n">
         <v>-7.633</v>
@@ -31590,7 +31590,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -31651,7 +31651,7 @@
         <v>1.786</v>
       </c>
       <c r="AI7" t="n">
-        <v>-2072.081999999995</v>
+        <v>-2072.081999999999</v>
       </c>
       <c r="AJ7" t="n">
         <v>-6.467</v>
@@ -31803,7 +31803,7 @@
         <v>2.198</v>
       </c>
       <c r="AI8" t="n">
-        <v>-5551.592999999999</v>
+        <v>-5551.593000000001</v>
       </c>
       <c r="AJ8" t="n">
         <v>0.38</v>
@@ -31864,7 +31864,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -32077,7 +32077,7 @@
         <v>1.383</v>
       </c>
       <c r="AI10" t="n">
-        <v>72159.24699999994</v>
+        <v>72159.24699999997</v>
       </c>
       <c r="AJ10" t="n">
         <v>-11.405</v>
@@ -32238,7 +32238,7 @@
         <v>1.248</v>
       </c>
       <c r="AI11" t="n">
-        <v>75182.47699999997</v>
+        <v>75182.47699999998</v>
       </c>
       <c r="AJ11" t="n">
         <v>-9.868</v>
@@ -32551,7 +32551,7 @@
         <v>1.212</v>
       </c>
       <c r="AI13" t="n">
-        <v>85041.65799999997</v>
+        <v>85041.658</v>
       </c>
       <c r="AJ13" t="n">
         <v>-9.567</v>
@@ -32612,7 +32612,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -32925,7 +32925,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -33980,7 +33980,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -34664,7 +34664,7 @@
         <v>0.912</v>
       </c>
       <c r="AI27" t="n">
-        <v>482308.4170000001</v>
+        <v>482308.417</v>
       </c>
       <c r="AJ27" t="n">
         <v>12.989</v>
@@ -34890,7 +34890,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -35337,7 +35337,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -35933,7 +35933,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -35994,7 +35994,7 @@
         <v>1.282</v>
       </c>
       <c r="AI36" t="n">
-        <v>-2093.93</v>
+        <v>-2093.930000000001</v>
       </c>
       <c r="AJ36" t="n">
         <v>0</v>
@@ -36055,7 +36055,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -36329,7 +36329,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -37095,7 +37095,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -37399,7 +37399,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -37895,7 +37895,7 @@
         <v>584740.964</v>
       </c>
       <c r="O49" t="n">
-        <v>57219.16100000001</v>
+        <v>57219.161</v>
       </c>
       <c r="P49" t="n">
         <v>1.932</v>
@@ -38108,7 +38108,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -38169,7 +38169,7 @@
         <v>1.207</v>
       </c>
       <c r="AI51" t="n">
-        <v>536.0379999999986</v>
+        <v>536.0379999999996</v>
       </c>
       <c r="AJ51" t="n">
         <v>-8.407999999999999</v>
@@ -38534,7 +38534,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -38595,7 +38595,7 @@
         <v>1.219</v>
       </c>
       <c r="AI54" t="n">
-        <v>-6843.675999999999</v>
+        <v>-6843.676</v>
       </c>
       <c r="AJ54" t="n">
         <v>-9.135999999999999</v>
@@ -38656,7 +38656,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -38836,7 +38836,7 @@
         <v>42408.00799999999</v>
       </c>
       <c r="O56" t="n">
-        <v>2554.764000000001</v>
+        <v>2554.764</v>
       </c>
       <c r="P56" t="n">
         <v>0.946</v>
@@ -38948,7 +38948,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -39128,7 +39128,7 @@
         <v>113076.542</v>
       </c>
       <c r="O58" t="n">
-        <v>89209.49699999999</v>
+        <v>89209.497</v>
       </c>
       <c r="P58" t="n">
         <v>14.805</v>
@@ -39252,7 +39252,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -39684,7 +39684,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -40119,7 +40119,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -40180,7 +40180,7 @@
         <v>1.506</v>
       </c>
       <c r="AI65" t="n">
-        <v>1097.082999999999</v>
+        <v>1097.083000000001</v>
       </c>
       <c r="AJ65" t="n">
         <v>3.244</v>
@@ -40530,7 +40530,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -40682,7 +40682,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -40986,7 +40986,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -41138,7 +41138,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -41782,7 +41782,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -42092,7 +42092,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -42375,7 +42375,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -42840,7 +42840,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -42901,7 +42901,7 @@
         <v>0.909</v>
       </c>
       <c r="AI83" t="n">
-        <v>20403.411</v>
+        <v>20403.41100000001</v>
       </c>
       <c r="AJ83" t="n">
         <v>-10.621</v>
@@ -43123,7 +43123,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -43701,7 +43701,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -43860,7 +43860,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -44031,7 +44031,7 @@
         <v>53049.641</v>
       </c>
       <c r="O92" t="n">
-        <v>-71627.23300000001</v>
+        <v>-71627.23299999999</v>
       </c>
       <c r="P92" t="n">
         <v>-22.759</v>
@@ -44532,7 +44532,7 @@
         <v>2.167</v>
       </c>
       <c r="AI95" t="n">
-        <v>-36336.33499999999</v>
+        <v>-36336.335</v>
       </c>
       <c r="AJ95" t="n">
         <v>7.502</v>
@@ -44593,7 +44593,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -44937,7 +44937,7 @@
         <v>1.218</v>
       </c>
       <c r="AI98" t="n">
-        <v>9206.203000000001</v>
+        <v>9206.203</v>
       </c>
       <c r="AJ98" t="n">
         <v>-4.209</v>
@@ -45007,7 +45007,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -45229,7 +45229,7 @@
         <v>1.52</v>
       </c>
       <c r="AI100" t="n">
-        <v>1044.137999999999</v>
+        <v>1044.137999999998</v>
       </c>
       <c r="AJ100" t="n">
         <v>-0.302</v>
@@ -45381,7 +45381,7 @@
         <v>2.243</v>
       </c>
       <c r="AI101" t="n">
-        <v>-7342.066000000003</v>
+        <v>-7342.066000000001</v>
       </c>
       <c r="AJ101" t="n">
         <v>1.12</v>
@@ -45898,7 +45898,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -46097,7 +46097,7 @@
         <v>10333.757</v>
       </c>
       <c r="O107" t="n">
-        <v>4585.812999999998</v>
+        <v>4585.813</v>
       </c>
       <c r="P107" t="n">
         <v>4.439</v>
@@ -46355,7 +46355,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -46623,7 +46623,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -46684,7 +46684,7 @@
         <v>1.53</v>
       </c>
       <c r="AI111" t="n">
-        <v>44447.072</v>
+        <v>44447.07199999999</v>
       </c>
       <c r="AJ111" t="n">
         <v>41.067</v>
@@ -47053,7 +47053,7 @@
         <v>43767.119108461</v>
       </c>
       <c r="O114" t="n">
-        <v>45040.483647395</v>
+        <v>45040.48364739501</v>
       </c>
       <c r="P114" t="n">
         <v>19.006</v>
@@ -47104,7 +47104,7 @@
         <v>1.727</v>
       </c>
       <c r="AI114" t="n">
-        <v>73880.39491509199</v>
+        <v>73880.39491509201</v>
       </c>
       <c r="AJ114" t="n">
         <v>13.551</v>
@@ -47848,7 +47848,7 @@
         <v>57104.9273618</v>
       </c>
       <c r="O119" t="n">
-        <v>-8354.105685278017</v>
+        <v>-8354.105685278011</v>
       </c>
       <c r="P119" t="n">
         <v>-2.587</v>
@@ -48319,7 +48319,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -48620,7 +48620,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -48894,7 +48894,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -49107,7 +49107,7 @@
         <v>3.214</v>
       </c>
       <c r="AI128" t="n">
-        <v>-448.712</v>
+        <v>-448.7119999999998</v>
       </c>
       <c r="AJ128" t="n">
         <v>-8.398</v>
@@ -49168,7 +49168,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -49692,7 +49692,7 @@
         <v>1.841</v>
       </c>
       <c r="AI133" t="n">
-        <v>-8415.234000000002</v>
+        <v>-8415.234</v>
       </c>
       <c r="AJ133" t="n">
         <v>-5.98</v>
@@ -50298,7 +50298,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -50527,7 +50527,7 @@
         <v>110803.352</v>
       </c>
       <c r="O140" t="n">
-        <v>84929.841</v>
+        <v>84929.84099999999</v>
       </c>
       <c r="P140" t="n">
         <v>12.871</v>
@@ -51391,7 +51391,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -51522,7 +51522,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -51668,7 +51668,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -52246,7 +52246,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -52696,7 +52696,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -52818,7 +52818,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -52970,7 +52970,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -53092,7 +53092,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -54048,7 +54048,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -54410,7 +54410,7 @@
         <v>1.628</v>
       </c>
       <c r="AI168" t="n">
-        <v>-95355.82799999998</v>
+        <v>-95355.82799999999</v>
       </c>
       <c r="AJ168" t="n">
         <v>-8.385</v>
@@ -54571,7 +54571,7 @@
         <v>1.553</v>
       </c>
       <c r="AI169" t="n">
-        <v>31803.23300000001</v>
+        <v>31803.233</v>
       </c>
       <c r="AJ169" t="n">
         <v>4.369</v>
@@ -54764,7 +54764,7 @@
         <v>1.392</v>
       </c>
       <c r="AI170" t="n">
-        <v>49624.19500000001</v>
+        <v>49624.19499999999</v>
       </c>
       <c r="AJ170" t="n">
         <v>9.231999999999999</v>
@@ -55253,7 +55253,7 @@
         <v>1.148</v>
       </c>
       <c r="AI173" t="n">
-        <v>47597.061</v>
+        <v>47597.06099999999</v>
       </c>
       <c r="AJ173" t="n">
         <v>12.611</v>
@@ -55645,7 +55645,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -55922,7 +55922,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -56044,7 +56044,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -56175,7 +56175,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -56236,7 +56236,7 @@
         <v>0.951</v>
       </c>
       <c r="AI180" t="n">
-        <v>786.7630000000008</v>
+        <v>786.7630000000004</v>
       </c>
       <c r="AJ180" t="n">
         <v>0.008999999999999999</v>
@@ -56306,7 +56306,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -56428,7 +56428,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -57180,7 +57180,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -57472,7 +57472,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -57746,7 +57746,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -57868,7 +57868,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -58020,7 +58020,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -58768,7 +58768,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -59051,7 +59051,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -59325,7 +59325,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -59599,7 +59599,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -59730,7 +59730,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -60095,7 +60095,7 @@
         <v>1.861</v>
       </c>
       <c r="AI207" t="n">
-        <v>18205.90499999999</v>
+        <v>18205.905</v>
       </c>
       <c r="AJ207" t="n">
         <v>-11.997</v>
@@ -60156,7 +60156,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -60430,7 +60430,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -61572,7 +61572,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -61767,7 +61767,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -61962,7 +61962,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -62640,7 +62640,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -62922,7 +62922,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -63897,7 +63897,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -64854,7 +64854,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -65322,7 +65322,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -65871,7 +65871,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -65937,7 +65937,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -66132,7 +66132,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -66849,7 +66849,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -67083,7 +67083,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -67668,7 +67668,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -68040,7 +68040,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -68106,7 +68106,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -68340,7 +68340,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -68664,7 +68664,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -69084,7 +69084,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -69453,7 +69453,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -69825,7 +69825,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -69930,7 +69930,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -70164,7 +70164,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -70269,7 +70269,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -70983,7 +70983,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -71265,7 +71265,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -71508,7 +71508,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -71919,7 +71919,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -72162,7 +72162,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -72615,7 +72615,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -72718,7 +72718,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -73348,7 +73348,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -73741,7 +73741,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -74500,7 +74500,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -74861,7 +74861,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -75056,7 +75056,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -76743,7 +76743,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -77097,7 +77097,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -77292,7 +77292,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -77487,7 +77487,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -78367,7 +78367,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -79472,7 +79472,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -79586,7 +79586,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -79691,7 +79691,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -80141,7 +80141,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -80603,7 +80603,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -80708,7 +80708,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -80813,7 +80813,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -80876,7 +80876,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -81944,7 +81944,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -83603,7 +83603,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -83846,7 +83846,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -83912,7 +83912,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -84026,7 +84026,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -84140,7 +84140,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -84206,7 +84206,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -84932,7 +84932,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -85223,7 +85223,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -85418,7 +85418,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -85484,7 +85484,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -85589,7 +85589,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -86330,7 +86330,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -86573,7 +86573,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -86768,7 +86768,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -86963,7 +86963,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -87077,7 +87077,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -87401,7 +87401,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -87596,7 +87596,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">

</xml_diff>

<commit_message>
Cap nhat ALM cac ma dang missing — Q2-2024 — 2026-09-18
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -38222,7 +38222,7 @@
       </c>
       <c r="BL51" t="inlineStr">
         <is>
-          <t>2026-09-18T14:50:29+07:00</t>
+          <t>2026-09-18T18:42:35+07:00</t>
         </is>
       </c>
     </row>
@@ -39252,7 +39252,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -39262,12 +39262,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H59" t="n">
@@ -39292,16 +39292,16 @@
         <v>109262.475</v>
       </c>
       <c r="O59" t="n">
-        <v>0</v>
+        <v>188322</v>
       </c>
       <c r="P59" t="n">
-        <v>0</v>
+        <v>30.158</v>
       </c>
       <c r="Q59" t="n">
-        <v>0</v>
+        <v>32.425</v>
       </c>
       <c r="R59" t="n">
-        <v>0</v>
+        <v>51.972</v>
       </c>
       <c r="AF59" t="n">
         <v>5.653</v>
@@ -39354,6 +39354,47 @@
       <c r="AV59" t="n">
         <v>-9.845000000000001</v>
       </c>
+      <c r="AW59" t="n">
+        <v>704344682</v>
+      </c>
+      <c r="AX59" t="n">
+        <v>855914052</v>
+      </c>
+      <c r="AY59" t="n">
+        <v>50440285</v>
+      </c>
+      <c r="AZ59" t="n">
+        <v>1275056</v>
+      </c>
+      <c r="BA59" t="n">
+        <v>51715341</v>
+      </c>
+      <c r="BB59" t="n">
+        <v>51851325</v>
+      </c>
+      <c r="BC59" t="n">
+        <v>135984</v>
+      </c>
+      <c r="BD59" t="n">
+        <v>7.342</v>
+      </c>
+      <c r="BE59" t="n">
+        <v>8281.829</v>
+      </c>
+      <c r="BF59" t="n">
+        <v>98155.47199999999</v>
+      </c>
+      <c r="BG59" t="n">
+        <v>257.42</v>
+      </c>
+      <c r="BH59" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="BI59" t="n">
+        <v>5171534.1</v>
+      </c>
       <c r="BJ59" t="inlineStr">
         <is>
           <t>Báo cáo tài chính hợp nhất quý 2 năm 2024 (đã soát xét)</t>
@@ -39366,7 +39407,7 @@
       </c>
       <c r="BL59" t="inlineStr">
         <is>
-          <t>2026-09-18T14:52:58+07:00</t>
+          <t>2026-09-18T18:44:26+07:00</t>
         </is>
       </c>
     </row>
@@ -42954,7 +42995,7 @@
       </c>
       <c r="BL83" t="inlineStr">
         <is>
-          <t>2026-09-18T14:58:58+07:00</t>
+          <t>2026-09-18T18:47:22+07:00</t>
         </is>
       </c>
     </row>
@@ -43875,7 +43916,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -43962,6 +44003,47 @@
       <c r="AV91" t="n">
         <v>-53.373</v>
       </c>
+      <c r="AW91" t="n">
+        <v>66583.122</v>
+      </c>
+      <c r="AX91" t="n">
+        <v>64169.958</v>
+      </c>
+      <c r="AY91" t="n">
+        <v>5413.161</v>
+      </c>
+      <c r="AZ91" t="n">
+        <v>-348.976</v>
+      </c>
+      <c r="BA91" t="n">
+        <v>5064.188</v>
+      </c>
+      <c r="BB91" t="n">
+        <v>5064.188</v>
+      </c>
+      <c r="BC91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD91" t="n">
+        <v>7.606</v>
+      </c>
+      <c r="BE91" t="n">
+        <v>1.714</v>
+      </c>
+      <c r="BF91" t="n">
+        <v>14.947</v>
+      </c>
+      <c r="BG91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH91" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="BI91" t="n">
+        <v>506.419</v>
+      </c>
       <c r="BJ91" t="inlineStr">
         <is>
           <t>Báo cáo tài chính hợp nhất quý 2 năm 2024 (đã soát xét)</t>
@@ -43974,7 +44056,7 @@
       </c>
       <c r="BL91" t="inlineStr">
         <is>
-          <t>2026-09-18T15:01:04+07:00</t>
+          <t>2026-09-18T18:49:47+07:00</t>
         </is>
       </c>
     </row>
@@ -45022,7 +45104,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H99" t="n">
@@ -45109,6 +45191,47 @@
       <c r="AV99" t="n">
         <v>-16.117</v>
       </c>
+      <c r="AW99" t="n">
+        <v>2436.669</v>
+      </c>
+      <c r="AX99" t="n">
+        <v>5757.617</v>
+      </c>
+      <c r="AY99" t="n">
+        <v>-3290.948</v>
+      </c>
+      <c r="AZ99" t="n">
+        <v>50.922</v>
+      </c>
+      <c r="BA99" t="n">
+        <v>-3240.026</v>
+      </c>
+      <c r="BB99" t="n">
+        <v>70.176</v>
+      </c>
+      <c r="BC99" t="n">
+        <v>3310.202</v>
+      </c>
+      <c r="BD99" t="n">
+        <v>-132.969</v>
+      </c>
+      <c r="BE99" t="n">
+        <v>-1.415</v>
+      </c>
+      <c r="BF99" t="n">
+        <v>0.414</v>
+      </c>
+      <c r="BG99" t="n">
+        <v>19.537</v>
+      </c>
+      <c r="BH99" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="BI99" t="n">
+        <v>-324.003</v>
+      </c>
       <c r="BJ99" t="inlineStr">
         <is>
           <t>Báo cáo tài chính hợp nhất quý 2 năm 2024 (đã soát xét)</t>
@@ -45121,7 +45244,7 @@
       </c>
       <c r="BL99" t="inlineStr">
         <is>
-          <t>2026-09-18T15:03:23+07:00</t>
+          <t>2026-09-18T18:52:23+07:00</t>
         </is>
       </c>
     </row>
@@ -51447,7 +51570,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H148" t="n">
@@ -51534,6 +51657,47 @@
       <c r="AV148" t="n">
         <v>10.578</v>
       </c>
+      <c r="AW148" t="n">
+        <v>57.276</v>
+      </c>
+      <c r="AX148" t="n">
+        <v>6159.743</v>
+      </c>
+      <c r="AY148" t="n">
+        <v>-408.755</v>
+      </c>
+      <c r="AZ148" t="n">
+        <v>-3773.406</v>
+      </c>
+      <c r="BA148" t="n">
+        <v>-2295.458</v>
+      </c>
+      <c r="BB148" t="n">
+        <v>7.201</v>
+      </c>
+      <c r="BC148" t="n">
+        <v>2302.659</v>
+      </c>
+      <c r="BD148" t="n">
+        <v>-4007.714</v>
+      </c>
+      <c r="BE148" t="n">
+        <v>-0.8179999999999999</v>
+      </c>
+      <c r="BF148" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="BG148" t="n">
+        <v>7.027</v>
+      </c>
+      <c r="BH148" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="BI148" t="n">
+        <v>-229.546</v>
+      </c>
       <c r="BJ148" t="inlineStr">
         <is>
           <t>Báo cáo tài chính hợp nhất quý 2 năm 2024 (đã soát xét)</t>
@@ -51546,7 +51710,7 @@
       </c>
       <c r="BL148" t="inlineStr">
         <is>
-          <t>2026-09-18T15:15:05+07:00</t>
+          <t>2026-09-18T18:55:11+07:00</t>
         </is>
       </c>
     </row>
@@ -56371,7 +56535,7 @@
       </c>
       <c r="BL180" t="inlineStr">
         <is>
-          <t>2026-09-18T15:26:58+07:00</t>
+          <t>2026-09-18T19:02:27+07:00</t>
         </is>
       </c>
     </row>
@@ -59737,7 +59901,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H204" t="n">
@@ -59824,6 +59988,47 @@
       <c r="AV204" t="n">
         <v>-14.733</v>
       </c>
+      <c r="AW204" t="n">
+        <v>42150.18</v>
+      </c>
+      <c r="AX204" t="n">
+        <v>41735.951</v>
+      </c>
+      <c r="AY204" t="n">
+        <v>-58.814</v>
+      </c>
+      <c r="AZ204" t="n">
+        <v>268.788</v>
+      </c>
+      <c r="BA204" t="n">
+        <v>683.0170000000001</v>
+      </c>
+      <c r="BB204" t="n">
+        <v>683.0170000000001</v>
+      </c>
+      <c r="BC204" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD204" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="BE204" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="BF204" t="n">
+        <v>1.781</v>
+      </c>
+      <c r="BG204" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH204" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="BI204" t="n">
+        <v>68.30200000000001</v>
+      </c>
       <c r="BJ204" t="inlineStr">
         <is>
           <t>Báo cáo tài chính hợp nhất quý 2 năm 2024 (đã soát xét)</t>
@@ -59836,7 +60041,7 @@
       </c>
       <c r="BL204" t="inlineStr">
         <is>
-          <t>2026-09-18T15:32:54+07:00</t>
+          <t>2026-09-18T19:04:54+07:00</t>
         </is>
       </c>
     </row>
@@ -67888,7 +68093,7 @@
       </c>
       <c r="CE51" t="inlineStr">
         <is>
-          <t>2026-09-18T14:50:29+07:00</t>
+          <t>2026-09-18T18:42:35+07:00</t>
         </is>
       </c>
     </row>
@@ -68787,7 +68992,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -68797,13 +69002,34 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>missing</t>
-        </is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>133137</v>
+      </c>
+      <c r="H59" t="n">
+        <v>37203</v>
+      </c>
+      <c r="I59" t="n">
+        <v>17982</v>
+      </c>
+      <c r="J59" t="n">
+        <v>14154</v>
+      </c>
+      <c r="K59" t="n">
+        <v>122061</v>
+      </c>
+      <c r="L59" t="n">
+        <v>97855</v>
+      </c>
+      <c r="M59" t="n">
+        <v>17645</v>
       </c>
       <c r="AB59" t="n">
         <v>-186493.134</v>
@@ -68877,6 +69103,33 @@
       <c r="AY59" t="n">
         <v>3.858</v>
       </c>
+      <c r="BU59" t="n">
+        <v>658535334</v>
+      </c>
+      <c r="BV59" t="n">
+        <v>806710365</v>
+      </c>
+      <c r="BW59" t="n">
+        <v>51824969</v>
+      </c>
+      <c r="BX59" t="n">
+        <v>44956347</v>
+      </c>
+      <c r="BY59" t="n">
+        <v>46367387</v>
+      </c>
+      <c r="BZ59" t="n">
+        <v>-135984</v>
+      </c>
+      <c r="CA59" t="n">
+        <v>23634</v>
+      </c>
+      <c r="CB59" t="n">
+        <v>2010140</v>
+      </c>
+      <c r="CC59" t="n">
+        <v>23149</v>
+      </c>
       <c r="CD59" t="inlineStr">
         <is>
           <t>Báo cáo tài chính hợp nhất quý 2 năm 2024 (đã soát xét)</t>
@@ -68884,7 +69137,7 @@
       </c>
       <c r="CE59" t="inlineStr">
         <is>
-          <t>2026-09-18T14:52:58+07:00</t>
+          <t>2026-09-18T18:44:26+07:00</t>
         </is>
       </c>
     </row>
@@ -72139,7 +72392,7 @@
       </c>
       <c r="CE83" t="inlineStr">
         <is>
-          <t>2026-09-18T14:58:58+07:00</t>
+          <t>2026-09-18T18:47:22+07:00</t>
         </is>
       </c>
     </row>
@@ -72856,7 +73109,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="AB91" t="n">
@@ -72931,6 +73184,33 @@
       <c r="AY91" t="n">
         <v>49130.755</v>
       </c>
+      <c r="BU91" t="n">
+        <v>32833.823</v>
+      </c>
+      <c r="BV91" t="n">
+        <v>30589.584</v>
+      </c>
+      <c r="BW91" t="n">
+        <v>881.3200000000001</v>
+      </c>
+      <c r="BX91" t="n">
+        <v>321.626</v>
+      </c>
+      <c r="BY91" t="n">
+        <v>1297.821</v>
+      </c>
+      <c r="BZ91" t="n">
+        <v>144.886</v>
+      </c>
+      <c r="CA91" t="n">
+        <v>136.112</v>
+      </c>
+      <c r="CB91" t="n">
+        <v>197.574</v>
+      </c>
+      <c r="CC91" t="n">
+        <v>5.888</v>
+      </c>
       <c r="CD91" t="inlineStr">
         <is>
           <t>Báo cáo tài chính hợp nhất quý 2 năm 2024 (đã soát xét)</t>
@@ -72938,7 +73218,7 @@
       </c>
       <c r="CE91" t="inlineStr">
         <is>
-          <t>2026-09-18T15:01:04+07:00</t>
+          <t>2026-09-18T18:49:47+07:00</t>
         </is>
       </c>
     </row>
@@ -73879,7 +74159,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="AB99" t="n">
@@ -73954,6 +74234,33 @@
       <c r="AY99" t="n">
         <v>471.129</v>
       </c>
+      <c r="BU99" t="n">
+        <v>2344.576</v>
+      </c>
+      <c r="BV99" t="n">
+        <v>5703.149</v>
+      </c>
+      <c r="BW99" t="n">
+        <v>-3310.202</v>
+      </c>
+      <c r="BX99" t="n">
+        <v>22.896</v>
+      </c>
+      <c r="BY99" t="n">
+        <v>6.989</v>
+      </c>
+      <c r="BZ99" t="n">
+        <v>15.907</v>
+      </c>
+      <c r="CA99" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB99" t="n">
+        <v>47.479</v>
+      </c>
+      <c r="CC99" t="n">
+        <v>2.551</v>
+      </c>
       <c r="CD99" t="inlineStr">
         <is>
           <t>Báo cáo tài chính hợp nhất quý 2 năm 2024 (đã soát xét)</t>
@@ -73961,7 +74268,7 @@
       </c>
       <c r="CE99" t="inlineStr">
         <is>
-          <t>2026-09-18T15:03:23+07:00</t>
+          <t>2026-09-18T18:52:23+07:00</t>
         </is>
       </c>
     </row>
@@ -79628,7 +79935,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="AB148" t="n">
@@ -79703,6 +80010,24 @@
       <c r="AY148" t="n">
         <v>5164.894</v>
       </c>
+      <c r="BU148" t="n">
+        <v>5.609</v>
+      </c>
+      <c r="BV148" t="n">
+        <v>6115.277</v>
+      </c>
+      <c r="BW148" t="n">
+        <v>-2302.659</v>
+      </c>
+      <c r="BX148" t="n">
+        <v>51.667</v>
+      </c>
+      <c r="BY148" t="n">
+        <v>44.466</v>
+      </c>
+      <c r="BZ148" t="n">
+        <v>7.201</v>
+      </c>
       <c r="CD148" t="inlineStr">
         <is>
           <t>Báo cáo tài chính hợp nhất quý 2 năm 2024 (đã soát xét)</t>
@@ -79710,7 +80035,7 @@
       </c>
       <c r="CE148" t="inlineStr">
         <is>
-          <t>2026-09-18T15:15:05+07:00</t>
+          <t>2026-09-18T18:55:11+07:00</t>
         </is>
       </c>
     </row>
@@ -84273,7 +84598,7 @@
       </c>
       <c r="CE180" t="inlineStr">
         <is>
-          <t>2026-09-18T15:26:58+07:00</t>
+          <t>2026-09-18T19:02:27+07:00</t>
         </is>
       </c>
     </row>
@@ -87155,7 +87480,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="AB204" t="n">
@@ -87230,6 +87555,24 @@
       <c r="AY204" t="n">
         <v>5529.611</v>
       </c>
+      <c r="BU204" t="n">
+        <v>41781.83</v>
+      </c>
+      <c r="BV204" t="n">
+        <v>41304.07</v>
+      </c>
+      <c r="BW204" t="n">
+        <v>678.342</v>
+      </c>
+      <c r="CA204" t="n">
+        <v>368.35</v>
+      </c>
+      <c r="CB204" t="n">
+        <v>431.881</v>
+      </c>
+      <c r="CC204" t="n">
+        <v>4.675</v>
+      </c>
       <c r="CD204" t="inlineStr">
         <is>
           <t>Báo cáo tài chính hợp nhất quý 2 năm 2024 (đã soát xét)</t>
@@ -87237,7 +87580,7 @@
       </c>
       <c r="CE204" t="inlineStr">
         <is>
-          <t>2026-09-18T15:32:54+07:00</t>
+          <t>2026-09-18T19:04:54+07:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cap nhat ALM cac ma dang missing — Q3-2024 — 2026-09-18
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -35558,7 +35558,7 @@
       </c>
       <c r="BL31" t="inlineStr">
         <is>
-          <t>2026-09-18T19:13:58+07:00</t>
+          <t>2026-09-18T20:55:56+07:00</t>
         </is>
       </c>
     </row>
@@ -46313,7 +46313,7 @@
       </c>
       <c r="BL103" t="inlineStr">
         <is>
-          <t>2026-09-18T19:24:17+07:00</t>
+          <t>2026-09-18T20:58:41+07:00</t>
         </is>
       </c>
     </row>
@@ -51779,7 +51779,7 @@
       </c>
       <c r="BL140" t="inlineStr">
         <is>
-          <t>2026-09-18T19:29:28+07:00</t>
+          <t>2026-09-18T21:00:21+07:00</t>
         </is>
       </c>
     </row>
@@ -52827,7 +52827,7 @@
       </c>
       <c r="BL149" t="inlineStr">
         <is>
-          <t>2026-09-18T19:30:51+07:00</t>
+          <t>2026-09-18T21:02:27+07:00</t>
         </is>
       </c>
     </row>
@@ -53881,7 +53881,7 @@
       </c>
       <c r="BL158" t="inlineStr">
         <is>
-          <t>2026-09-18T19:31:22+07:00</t>
+          <t>2026-09-18T21:03:12+07:00</t>
         </is>
       </c>
     </row>
@@ -54968,7 +54968,7 @@
       </c>
       <c r="BL167" t="inlineStr">
         <is>
-          <t>2026-09-18T19:33:04+07:00</t>
+          <t>2026-09-18T21:05:47+07:00</t>
         </is>
       </c>
     </row>
@@ -60504,7 +60504,7 @@
       </c>
       <c r="BL203" t="inlineStr">
         <is>
-          <t>2026-09-18T19:39:32+07:00</t>
+          <t>2026-09-18T21:08:45+07:00</t>
         </is>
       </c>
     </row>
@@ -64416,7 +64416,7 @@
       </c>
       <c r="BL230" t="inlineStr">
         <is>
-          <t>2026-09-18T19:41:51+07:00</t>
+          <t>2026-09-18T21:08:49+07:00</t>
         </is>
       </c>
     </row>
@@ -70113,7 +70113,7 @@
       </c>
       <c r="CE31" t="inlineStr">
         <is>
-          <t>2026-09-18T19:13:58+07:00</t>
+          <t>2026-09-18T20:55:56+07:00</t>
         </is>
       </c>
     </row>
@@ -79933,7 +79933,7 @@
       </c>
       <c r="CE103" t="inlineStr">
         <is>
-          <t>2026-09-18T19:24:17+07:00</t>
+          <t>2026-09-18T20:58:41+07:00</t>
         </is>
       </c>
     </row>
@@ -85080,7 +85080,7 @@
       </c>
       <c r="CE140" t="inlineStr">
         <is>
-          <t>2026-09-18T19:29:28+07:00</t>
+          <t>2026-09-18T21:00:21+07:00</t>
         </is>
       </c>
     </row>
@@ -85868,7 +85868,7 @@
       </c>
       <c r="CE149" t="inlineStr">
         <is>
-          <t>2026-09-18T19:30:51+07:00</t>
+          <t>2026-09-18T21:02:27+07:00</t>
         </is>
       </c>
     </row>
@@ -86764,7 +86764,7 @@
       </c>
       <c r="CE158" t="inlineStr">
         <is>
-          <t>2026-09-18T19:31:22+07:00</t>
+          <t>2026-09-18T21:03:12+07:00</t>
         </is>
       </c>
     </row>
@@ -87793,7 +87793,7 @@
       </c>
       <c r="CE167" t="inlineStr">
         <is>
-          <t>2026-09-18T19:33:04+07:00</t>
+          <t>2026-09-18T21:05:47+07:00</t>
         </is>
       </c>
     </row>
@@ -93160,7 +93160,7 @@
       </c>
       <c r="CE203" t="inlineStr">
         <is>
-          <t>2026-09-18T19:39:32+07:00</t>
+          <t>2026-09-18T21:08:45+07:00</t>
         </is>
       </c>
     </row>
@@ -96602,7 +96602,7 @@
       </c>
       <c r="CE230" t="inlineStr">
         <is>
-          <t>2026-09-18T19:41:51+07:00</t>
+          <t>2026-09-18T21:08:49+07:00</t>
         </is>
       </c>
     </row>

</xml_diff>